<commit_message>
fix: preserve sheetProtection in LLP Incertidumbre sheet
</commit_message>
<xml_diff>
--- a/app/templates/informes/LLP/1-INF.-N-000-26-SU23-LL-LP-V07.xlsx
+++ b/app/templates/informes/LLP/1-INF.-N-000-26-SU23-LL-LP-V07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\LLP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3915625E-7050-4D49-A157-AAA31E5D4D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79D023E-EDD6-49DD-A89E-7FE6478C4C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="737" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5385,6 +5385,54 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
@@ -5405,15 +5453,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5475,216 +5514,51 @@
     <xf numFmtId="167" fontId="28" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="23" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="23" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="191" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="11" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="50" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5714,39 +5588,223 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="191" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="11" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="1" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="190" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="187" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="60" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -5778,63 +5836,34 @@
     <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="187" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="60" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="1" xfId="21" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="190" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="78" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5857,35 +5886,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="2" borderId="20" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5955,14 +5955,36 @@
     <xf numFmtId="0" fontId="56" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="66" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="66" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5971,28 +5993,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -12891,35 +12891,35 @@
     </row>
     <row r="6" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="790" t="s">
+      <c r="A7" s="802" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="790"/>
-      <c r="C7" s="790"/>
-      <c r="D7" s="790"/>
-      <c r="E7" s="790"/>
-      <c r="F7" s="790"/>
-      <c r="G7" s="790"/>
-      <c r="H7" s="790"/>
-      <c r="I7" s="790"/>
-      <c r="J7" s="790"/>
-      <c r="K7" s="790"/>
+      <c r="B7" s="802"/>
+      <c r="C7" s="802"/>
+      <c r="D7" s="802"/>
+      <c r="E7" s="802"/>
+      <c r="F7" s="802"/>
+      <c r="G7" s="802"/>
+      <c r="H7" s="802"/>
+      <c r="I7" s="802"/>
+      <c r="J7" s="802"/>
+      <c r="K7" s="802"/>
     </row>
     <row r="8" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="782">
+      <c r="A8" s="797">
         <f>+K13</f>
         <v>10</v>
       </c>
-      <c r="B8" s="782"/>
-      <c r="C8" s="782"/>
-      <c r="D8" s="782"/>
-      <c r="E8" s="782"/>
-      <c r="F8" s="782"/>
-      <c r="G8" s="782"/>
-      <c r="H8" s="782"/>
-      <c r="I8" s="782"/>
-      <c r="J8" s="782"/>
-      <c r="K8" s="782"/>
+      <c r="B8" s="797"/>
+      <c r="C8" s="797"/>
+      <c r="D8" s="797"/>
+      <c r="E8" s="797"/>
+      <c r="F8" s="797"/>
+      <c r="G8" s="797"/>
+      <c r="H8" s="797"/>
+      <c r="I8" s="797"/>
+      <c r="J8" s="797"/>
+      <c r="K8" s="797"/>
     </row>
     <row r="9" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O9" s="26"/>
@@ -13030,8 +13030,8 @@
       <c r="M13" s="32"/>
       <c r="P13" s="36"/>
       <c r="Q13" s="36"/>
-      <c r="R13" s="797"/>
-      <c r="S13" s="797"/>
+      <c r="R13" s="809"/>
+      <c r="S13" s="809"/>
     </row>
     <row r="14" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="148" t="s">
@@ -13055,19 +13055,19 @@
       <c r="S14" s="42"/>
     </row>
     <row r="15" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="798" t="s">
+      <c r="A15" s="810" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="799"/>
-      <c r="C15" s="799"/>
-      <c r="D15" s="799"/>
-      <c r="E15" s="799"/>
-      <c r="F15" s="799"/>
-      <c r="G15" s="799"/>
-      <c r="H15" s="799"/>
-      <c r="I15" s="799"/>
-      <c r="J15" s="799"/>
-      <c r="K15" s="800"/>
+      <c r="B15" s="811"/>
+      <c r="C15" s="811"/>
+      <c r="D15" s="811"/>
+      <c r="E15" s="811"/>
+      <c r="F15" s="811"/>
+      <c r="G15" s="811"/>
+      <c r="H15" s="811"/>
+      <c r="I15" s="811"/>
+      <c r="J15" s="811"/>
+      <c r="K15" s="812"/>
       <c r="L15" s="32"/>
       <c r="M15" s="32"/>
       <c r="P15" s="36"/>
@@ -13076,19 +13076,19 @@
       <c r="S15" s="42"/>
     </row>
     <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="802" t="s">
+      <c r="A16" s="814" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="803"/>
-      <c r="C16" s="803"/>
-      <c r="D16" s="803"/>
-      <c r="E16" s="803"/>
-      <c r="F16" s="803"/>
-      <c r="G16" s="803"/>
-      <c r="H16" s="803"/>
-      <c r="I16" s="803"/>
-      <c r="J16" s="803"/>
-      <c r="K16" s="804"/>
+      <c r="B16" s="815"/>
+      <c r="C16" s="815"/>
+      <c r="D16" s="815"/>
+      <c r="E16" s="815"/>
+      <c r="F16" s="815"/>
+      <c r="G16" s="815"/>
+      <c r="H16" s="815"/>
+      <c r="I16" s="815"/>
+      <c r="J16" s="815"/>
+      <c r="K16" s="816"/>
       <c r="L16" s="32"/>
       <c r="M16" s="32"/>
       <c r="N16" s="23" t="s">
@@ -13100,10 +13100,10 @@
       <c r="S16" s="42"/>
     </row>
     <row r="17" spans="1:30" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="783" t="s">
+      <c r="A17" s="798" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="784"/>
+      <c r="B17" s="799"/>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="44"/>
@@ -13148,8 +13148,8 @@
       <c r="AD17" s="118"/>
     </row>
     <row r="18" spans="1:30" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="785"/>
-      <c r="B18" s="786"/>
+      <c r="A18" s="800"/>
+      <c r="B18" s="801"/>
       <c r="C18" s="145"/>
       <c r="D18" s="145"/>
       <c r="E18" s="145"/>
@@ -13301,10 +13301,10 @@
       <c r="T20" s="128" t="s">
         <v>50</v>
       </c>
-      <c r="U20" s="781">
+      <c r="U20" s="796">
         <v>44090</v>
       </c>
-      <c r="V20" s="781"/>
+      <c r="V20" s="796"/>
       <c r="W20" s="129"/>
       <c r="X20" s="130"/>
       <c r="Y20" s="129"/>
@@ -13398,8 +13398,8 @@
     </row>
     <row r="23" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="52"/>
-      <c r="I23" s="791"/>
-      <c r="J23" s="791"/>
+      <c r="I23" s="803"/>
+      <c r="J23" s="803"/>
       <c r="K23" s="53"/>
       <c r="L23" s="32"/>
       <c r="M23" s="54"/>
@@ -13407,44 +13407,44 @@
     </row>
     <row r="24" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="56"/>
-      <c r="D24" s="793" t="s">
+      <c r="D24" s="805" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="794"/>
-      <c r="F24" s="794"/>
-      <c r="G24" s="795" t="s">
+      <c r="E24" s="806"/>
+      <c r="F24" s="806"/>
+      <c r="G24" s="807" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="796"/>
-      <c r="I24" s="792"/>
-      <c r="J24" s="792"/>
+      <c r="H24" s="808"/>
+      <c r="I24" s="804"/>
+      <c r="J24" s="804"/>
       <c r="K24" s="57"/>
       <c r="L24" s="32"/>
       <c r="M24" s="58"/>
       <c r="N24" s="138" t="s">
         <v>52</v>
       </c>
-      <c r="O24" s="805" t="s">
+      <c r="O24" s="817" t="s">
         <v>35</v>
       </c>
-      <c r="P24" s="807"/>
+      <c r="P24" s="819"/>
       <c r="Q24" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="R24" s="805" t="s">
+      <c r="R24" s="817" t="s">
         <v>34</v>
       </c>
-      <c r="S24" s="806"/>
+      <c r="S24" s="818"/>
       <c r="T24" s="59" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="808" t="s">
+      <c r="A25" s="793" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="809"/>
-      <c r="C25" s="810"/>
+      <c r="B25" s="794"/>
+      <c r="C25" s="795"/>
       <c r="D25" s="60">
         <f>IF($Q$24="NO","",O25)</f>
         <v>1</v>
@@ -13465,8 +13465,8 @@
         <f>IF($T$24="NO","",S25)</f>
         <v>2</v>
       </c>
-      <c r="I25" s="792"/>
-      <c r="J25" s="792"/>
+      <c r="I25" s="804"/>
+      <c r="J25" s="804"/>
       <c r="K25" s="57"/>
       <c r="L25" s="32"/>
       <c r="M25" s="58"/>
@@ -13490,11 +13490,11 @@
       </c>
     </row>
     <row r="26" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="787" t="s">
+      <c r="A26" s="790" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="788"/>
-      <c r="C26" s="789"/>
+      <c r="B26" s="791"/>
+      <c r="C26" s="792"/>
       <c r="D26" s="66">
         <f>IF($Q$24="NO","",O26)</f>
         <v>5</v>
@@ -13515,8 +13515,8 @@
         <f>IF($T$24="NO","",S26)</f>
         <v>10</v>
       </c>
-      <c r="I26" s="801"/>
-      <c r="J26" s="801"/>
+      <c r="I26" s="813"/>
+      <c r="J26" s="813"/>
       <c r="K26" s="69"/>
       <c r="L26" s="70"/>
       <c r="M26" s="58"/>
@@ -13545,11 +13545,11 @@
       </c>
     </row>
     <row r="27" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="787" t="s">
+      <c r="A27" s="790" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="788"/>
-      <c r="C27" s="789"/>
+      <c r="B27" s="791"/>
+      <c r="C27" s="792"/>
       <c r="D27" s="66">
         <f t="shared" ref="D27:D29" si="2">IF($Q$24="NO","",O27)</f>
         <v>34</v>
@@ -13588,11 +13588,11 @@
       <c r="S27" s="136"/>
     </row>
     <row r="28" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="787" t="s">
+      <c r="A28" s="790" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="788"/>
-      <c r="C28" s="789"/>
+      <c r="B28" s="791"/>
+      <c r="C28" s="792"/>
       <c r="D28" s="86">
         <f t="shared" si="2"/>
         <v>45.749976347249998</v>
@@ -13643,11 +13643,11 @@
       </c>
     </row>
     <row r="29" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="787" t="s">
+      <c r="A29" s="790" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="788"/>
-      <c r="C29" s="789"/>
+      <c r="B29" s="791"/>
+      <c r="C29" s="792"/>
       <c r="D29" s="86">
         <f t="shared" si="2"/>
         <v>41.369978611709996</v>
@@ -13698,11 +13698,11 @@
       </c>
     </row>
     <row r="30" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="787" t="s">
+      <c r="A30" s="790" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="788"/>
-      <c r="C30" s="789"/>
+      <c r="B30" s="791"/>
+      <c r="C30" s="792"/>
       <c r="D30" s="86">
         <f t="shared" ref="D30:F33" si="10">IF($Q$24="NO","",O31)</f>
         <v>22.739988243419997</v>
@@ -13753,11 +13753,11 @@
       </c>
     </row>
     <row r="31" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="787" t="s">
+      <c r="A31" s="790" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="788"/>
-      <c r="C31" s="789"/>
+      <c r="B31" s="791"/>
+      <c r="C31" s="792"/>
       <c r="D31" s="86">
         <f t="shared" si="10"/>
         <v>4.3799977355400017</v>
@@ -13808,11 +13808,11 @@
       </c>
     </row>
     <row r="32" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="787" t="s">
+      <c r="A32" s="790" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="788"/>
-      <c r="C32" s="789"/>
+      <c r="B32" s="791"/>
+      <c r="C32" s="792"/>
       <c r="D32" s="86">
         <f t="shared" si="10"/>
         <v>18.629990368289999</v>
@@ -13863,11 +13863,11 @@
       </c>
     </row>
     <row r="33" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="808" t="s">
+      <c r="A33" s="793" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="809"/>
-      <c r="C33" s="810"/>
+      <c r="B33" s="794"/>
+      <c r="C33" s="795"/>
       <c r="D33" s="86">
         <f t="shared" si="10"/>
         <v>23.510466988727867</v>
@@ -13977,10 +13977,10 @@
       <c r="D36" s="17"/>
       <c r="E36" s="17"/>
       <c r="F36" s="17"/>
-      <c r="G36" s="811" t="s">
+      <c r="G36" s="781" t="s">
         <v>75</v>
       </c>
-      <c r="H36" s="812"/>
+      <c r="H36" s="782"/>
       <c r="I36" s="152">
         <f>+IF(Q24="NO","NP",ROUND(O49,0))</f>
         <v>24</v>
@@ -14034,10 +14034,10 @@
       <c r="D38" s="17"/>
       <c r="E38" s="17"/>
       <c r="F38" s="17"/>
-      <c r="G38" s="811" t="s">
+      <c r="G38" s="781" t="s">
         <v>76</v>
       </c>
-      <c r="H38" s="812"/>
+      <c r="H38" s="782"/>
       <c r="I38" s="152">
         <f>+IF(T24="NO","NP",ROUND(O42,0))</f>
         <v>13</v>
@@ -14089,10 +14089,10 @@
       <c r="D40" s="19"/>
       <c r="E40" s="19"/>
       <c r="F40" s="19"/>
-      <c r="G40" s="811" t="s">
+      <c r="G40" s="781" t="s">
         <v>77</v>
       </c>
-      <c r="H40" s="812"/>
+      <c r="H40" s="782"/>
       <c r="I40" s="152">
         <f>IF(T24="NO","NP",I36-I38)</f>
         <v>11</v>
@@ -14474,12 +14474,12 @@
       <c r="E57" s="168"/>
       <c r="F57" s="169"/>
       <c r="G57" s="169"/>
-      <c r="H57" s="816" t="s">
+      <c r="H57" s="786" t="s">
         <v>101</v>
       </c>
-      <c r="I57" s="817"/>
-      <c r="J57" s="817"/>
-      <c r="K57" s="818"/>
+      <c r="I57" s="787"/>
+      <c r="J57" s="787"/>
+      <c r="K57" s="788"/>
       <c r="L57" s="32"/>
       <c r="M57" s="32"/>
     </row>
@@ -14493,31 +14493,31 @@
       <c r="E58" s="168"/>
       <c r="F58" s="169"/>
       <c r="G58" s="169"/>
-      <c r="H58" s="816" t="s">
+      <c r="H58" s="786" t="s">
         <v>102</v>
       </c>
-      <c r="I58" s="817"/>
-      <c r="J58" s="817"/>
-      <c r="K58" s="818"/>
+      <c r="I58" s="787"/>
+      <c r="J58" s="787"/>
+      <c r="K58" s="788"/>
       <c r="L58" s="32"/>
       <c r="M58" s="32"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="815" t="s">
+      <c r="A59" s="785" t="s">
         <v>84</v>
       </c>
-      <c r="B59" s="815"/>
-      <c r="C59" s="815"/>
-      <c r="D59" s="815"/>
-      <c r="E59" s="815"/>
-      <c r="F59" s="815"/>
-      <c r="G59" s="815"/>
-      <c r="H59" s="816">
+      <c r="B59" s="785"/>
+      <c r="C59" s="785"/>
+      <c r="D59" s="785"/>
+      <c r="E59" s="785"/>
+      <c r="F59" s="785"/>
+      <c r="G59" s="785"/>
+      <c r="H59" s="786">
         <v>23</v>
       </c>
-      <c r="I59" s="817"/>
-      <c r="J59" s="817"/>
-      <c r="K59" s="818"/>
+      <c r="I59" s="787"/>
+      <c r="J59" s="787"/>
+      <c r="K59" s="788"/>
       <c r="L59" s="32"/>
       <c r="M59" s="32"/>
       <c r="N59" s="153"/>
@@ -14532,31 +14532,31 @@
       <c r="E60" s="168"/>
       <c r="F60" s="169"/>
       <c r="G60" s="169"/>
-      <c r="H60" s="816" t="s">
+      <c r="H60" s="786" t="s">
         <v>103</v>
       </c>
-      <c r="I60" s="817"/>
-      <c r="J60" s="817"/>
-      <c r="K60" s="818"/>
+      <c r="I60" s="787"/>
+      <c r="J60" s="787"/>
+      <c r="K60" s="788"/>
       <c r="L60" s="32"/>
       <c r="M60" s="32"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="815" t="s">
+      <c r="A61" s="785" t="s">
         <v>86</v>
       </c>
-      <c r="B61" s="815"/>
-      <c r="C61" s="815"/>
-      <c r="D61" s="815"/>
-      <c r="E61" s="815"/>
-      <c r="F61" s="815"/>
-      <c r="G61" s="815"/>
-      <c r="H61" s="816" t="s">
+      <c r="B61" s="785"/>
+      <c r="C61" s="785"/>
+      <c r="D61" s="785"/>
+      <c r="E61" s="785"/>
+      <c r="F61" s="785"/>
+      <c r="G61" s="785"/>
+      <c r="H61" s="786" t="s">
         <v>104</v>
       </c>
-      <c r="I61" s="817"/>
-      <c r="J61" s="817"/>
-      <c r="K61" s="818"/>
+      <c r="I61" s="787"/>
+      <c r="J61" s="787"/>
+      <c r="K61" s="788"/>
       <c r="L61" s="32"/>
       <c r="M61" s="32"/>
     </row>
@@ -14586,13 +14586,13 @@
       <c r="B64" s="156"/>
       <c r="C64" s="156"/>
       <c r="D64" s="156"/>
-      <c r="H64" s="819"/>
-      <c r="I64" s="819"/>
-      <c r="J64" s="819"/>
-      <c r="K64" s="819"/>
-      <c r="L64" s="819"/>
-      <c r="M64" s="819"/>
-      <c r="N64" s="819"/>
+      <c r="H64" s="789"/>
+      <c r="I64" s="789"/>
+      <c r="J64" s="789"/>
+      <c r="K64" s="789"/>
+      <c r="L64" s="789"/>
+      <c r="M64" s="789"/>
+      <c r="N64" s="789"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="157" t="s">
@@ -14654,12 +14654,12 @@
       </c>
       <c r="B71" s="160"/>
       <c r="D71" s="161"/>
-      <c r="H71" s="814" t="s">
+      <c r="H71" s="784" t="s">
         <v>81</v>
       </c>
-      <c r="I71" s="814"/>
-      <c r="J71" s="814"/>
-      <c r="K71" s="814"/>
+      <c r="I71" s="784"/>
+      <c r="J71" s="784"/>
+      <c r="K71" s="784"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="18"/>
@@ -14679,32 +14679,32 @@
       </c>
     </row>
     <row r="75" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="813" t="s">
+      <c r="A75" s="783" t="s">
         <v>79</v>
       </c>
-      <c r="B75" s="813"/>
-      <c r="C75" s="813"/>
-      <c r="D75" s="813"/>
-      <c r="E75" s="813"/>
-      <c r="F75" s="813"/>
-      <c r="G75" s="813"/>
-      <c r="H75" s="813"/>
-      <c r="I75" s="813"/>
-      <c r="J75" s="813"/>
-      <c r="K75" s="813"/>
+      <c r="B75" s="783"/>
+      <c r="C75" s="783"/>
+      <c r="D75" s="783"/>
+      <c r="E75" s="783"/>
+      <c r="F75" s="783"/>
+      <c r="G75" s="783"/>
+      <c r="H75" s="783"/>
+      <c r="I75" s="783"/>
+      <c r="J75" s="783"/>
+      <c r="K75" s="783"/>
     </row>
     <row r="76" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="813"/>
-      <c r="B76" s="813"/>
-      <c r="C76" s="813"/>
-      <c r="D76" s="813"/>
-      <c r="E76" s="813"/>
-      <c r="F76" s="813"/>
-      <c r="G76" s="813"/>
-      <c r="H76" s="813"/>
-      <c r="I76" s="813"/>
-      <c r="J76" s="813"/>
-      <c r="K76" s="813"/>
+      <c r="A76" s="783"/>
+      <c r="B76" s="783"/>
+      <c r="C76" s="783"/>
+      <c r="D76" s="783"/>
+      <c r="E76" s="783"/>
+      <c r="F76" s="783"/>
+      <c r="G76" s="783"/>
+      <c r="H76" s="783"/>
+      <c r="I76" s="783"/>
+      <c r="J76" s="783"/>
+      <c r="K76" s="783"/>
     </row>
     <row r="78" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -14713,28 +14713,6 @@
     <protectedRange sqref="C10:C11" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="38">
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="A76:K76"/>
-    <mergeCell ref="H71:K71"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="H57:K57"/>
-    <mergeCell ref="H59:K59"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="H64:N64"/>
-    <mergeCell ref="H58:K58"/>
-    <mergeCell ref="H60:K60"/>
-    <mergeCell ref="H61:K61"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
     <mergeCell ref="U20:V20"/>
     <mergeCell ref="A8:K8"/>
     <mergeCell ref="A17:B18"/>
@@ -14751,6 +14729,28 @@
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="R24:S24"/>
     <mergeCell ref="O24:P24"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="H71:K71"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="H57:K57"/>
+    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="H64:N64"/>
+    <mergeCell ref="H58:K58"/>
+    <mergeCell ref="H60:K60"/>
+    <mergeCell ref="H61:K61"/>
   </mergeCells>
   <conditionalFormatting sqref="A59">
     <cfRule type="cellIs" priority="2" stopIfTrue="1" operator="between">
@@ -14909,42 +14909,42 @@
       <c r="Q6" s="770"/>
     </row>
     <row r="7" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="823" t="s">
+      <c r="A7" s="881" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="823"/>
-      <c r="C7" s="823"/>
-      <c r="D7" s="823"/>
-      <c r="E7" s="823"/>
-      <c r="F7" s="823"/>
-      <c r="G7" s="823"/>
-      <c r="H7" s="823"/>
-      <c r="I7" s="823"/>
-      <c r="J7" s="823"/>
-      <c r="K7" s="823"/>
-      <c r="L7" s="823"/>
-      <c r="M7" s="823"/>
+      <c r="B7" s="881"/>
+      <c r="C7" s="881"/>
+      <c r="D7" s="881"/>
+      <c r="E7" s="881"/>
+      <c r="F7" s="881"/>
+      <c r="G7" s="881"/>
+      <c r="H7" s="881"/>
+      <c r="I7" s="881"/>
+      <c r="J7" s="881"/>
+      <c r="K7" s="881"/>
+      <c r="L7" s="881"/>
+      <c r="M7" s="881"/>
       <c r="P7" s="682" t="s">
         <v>269</v>
       </c>
       <c r="Q7" s="770"/>
     </row>
     <row r="8" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="824" t="s">
+      <c r="A8" s="882" t="s">
         <v>272</v>
       </c>
-      <c r="B8" s="824"/>
-      <c r="C8" s="824"/>
-      <c r="D8" s="824"/>
-      <c r="E8" s="824"/>
-      <c r="F8" s="824"/>
-      <c r="G8" s="824"/>
-      <c r="H8" s="824"/>
-      <c r="I8" s="824"/>
-      <c r="J8" s="824"/>
-      <c r="K8" s="824"/>
-      <c r="L8" s="824"/>
-      <c r="M8" s="824"/>
+      <c r="B8" s="882"/>
+      <c r="C8" s="882"/>
+      <c r="D8" s="882"/>
+      <c r="E8" s="882"/>
+      <c r="F8" s="882"/>
+      <c r="G8" s="882"/>
+      <c r="H8" s="882"/>
+      <c r="I8" s="882"/>
+      <c r="J8" s="882"/>
+      <c r="K8" s="882"/>
+      <c r="L8" s="882"/>
+      <c r="M8" s="882"/>
       <c r="P8" s="682" t="s">
         <v>319</v>
       </c>
@@ -14971,23 +14971,23 @@
     </row>
     <row r="10" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="679"/>
-      <c r="C10" s="825" t="s">
+      <c r="C10" s="883" t="s">
         <v>273</v>
       </c>
-      <c r="D10" s="825"/>
-      <c r="E10" s="825" t="s">
+      <c r="D10" s="883"/>
+      <c r="E10" s="883" t="s">
         <v>274</v>
       </c>
-      <c r="F10" s="825"/>
-      <c r="G10" s="825"/>
-      <c r="H10" s="825" t="s">
+      <c r="F10" s="883"/>
+      <c r="G10" s="883"/>
+      <c r="H10" s="883" t="s">
         <v>275</v>
       </c>
-      <c r="I10" s="825"/>
-      <c r="J10" s="825" t="s">
+      <c r="I10" s="883"/>
+      <c r="J10" s="883" t="s">
         <v>276</v>
       </c>
-      <c r="K10" s="825"/>
+      <c r="K10" s="883"/>
       <c r="L10" s="679"/>
       <c r="M10" s="679"/>
       <c r="N10" s="121"/>
@@ -14998,15 +14998,15 @@
     <row r="11" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="679"/>
       <c r="B11" s="679"/>
-      <c r="C11" s="826"/>
-      <c r="D11" s="826"/>
-      <c r="E11" s="826"/>
-      <c r="F11" s="826"/>
-      <c r="G11" s="826"/>
-      <c r="H11" s="827"/>
-      <c r="I11" s="826"/>
-      <c r="J11" s="826"/>
-      <c r="K11" s="826"/>
+      <c r="C11" s="884"/>
+      <c r="D11" s="884"/>
+      <c r="E11" s="884"/>
+      <c r="F11" s="884"/>
+      <c r="G11" s="884"/>
+      <c r="H11" s="885"/>
+      <c r="I11" s="884"/>
+      <c r="J11" s="884"/>
+      <c r="K11" s="884"/>
       <c r="L11" s="679"/>
       <c r="M11" s="679"/>
       <c r="N11" s="121"/>
@@ -15038,21 +15038,21 @@
       <c r="Q12" s="771"/>
     </row>
     <row r="13" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="828" t="s">
+      <c r="A13" s="886" t="s">
         <v>277</v>
       </c>
-      <c r="B13" s="829"/>
-      <c r="C13" s="829"/>
-      <c r="D13" s="829"/>
-      <c r="E13" s="829"/>
-      <c r="F13" s="829"/>
-      <c r="G13" s="829"/>
-      <c r="H13" s="829"/>
-      <c r="I13" s="829"/>
-      <c r="J13" s="829"/>
-      <c r="K13" s="829"/>
-      <c r="L13" s="829"/>
-      <c r="M13" s="830"/>
+      <c r="B13" s="887"/>
+      <c r="C13" s="887"/>
+      <c r="D13" s="887"/>
+      <c r="E13" s="887"/>
+      <c r="F13" s="887"/>
+      <c r="G13" s="887"/>
+      <c r="H13" s="887"/>
+      <c r="I13" s="887"/>
+      <c r="J13" s="887"/>
+      <c r="K13" s="887"/>
+      <c r="L13" s="887"/>
+      <c r="M13" s="888"/>
       <c r="N13" s="121"/>
       <c r="O13" s="121"/>
       <c r="P13" s="682" t="s">
@@ -15061,21 +15061,21 @@
       <c r="Q13" s="771"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="820" t="s">
+      <c r="A14" s="878" t="s">
         <v>236</v>
       </c>
-      <c r="B14" s="821"/>
-      <c r="C14" s="821"/>
-      <c r="D14" s="821"/>
-      <c r="E14" s="821"/>
-      <c r="F14" s="821"/>
-      <c r="G14" s="821"/>
-      <c r="H14" s="821"/>
-      <c r="I14" s="821"/>
-      <c r="J14" s="821"/>
-      <c r="K14" s="821"/>
-      <c r="L14" s="821"/>
-      <c r="M14" s="822"/>
+      <c r="B14" s="879"/>
+      <c r="C14" s="879"/>
+      <c r="D14" s="879"/>
+      <c r="E14" s="879"/>
+      <c r="F14" s="879"/>
+      <c r="G14" s="879"/>
+      <c r="H14" s="879"/>
+      <c r="I14" s="879"/>
+      <c r="J14" s="879"/>
+      <c r="K14" s="879"/>
+      <c r="L14" s="879"/>
+      <c r="M14" s="880"/>
       <c r="N14" s="121"/>
       <c r="O14" s="121"/>
       <c r="P14" s="769"/>
@@ -15103,19 +15103,19 @@
       <c r="Q15" s="772"/>
     </row>
     <row r="16" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="832" t="s">
+      <c r="B16" s="860" t="s">
         <v>218</v>
       </c>
-      <c r="C16" s="833"/>
-      <c r="D16" s="833"/>
-      <c r="E16" s="833"/>
-      <c r="F16" s="833"/>
-      <c r="G16" s="833"/>
-      <c r="H16" s="833"/>
-      <c r="I16" s="833"/>
-      <c r="J16" s="833"/>
-      <c r="K16" s="833"/>
-      <c r="L16" s="834"/>
+      <c r="C16" s="861"/>
+      <c r="D16" s="861"/>
+      <c r="E16" s="861"/>
+      <c r="F16" s="861"/>
+      <c r="G16" s="861"/>
+      <c r="H16" s="861"/>
+      <c r="I16" s="861"/>
+      <c r="J16" s="861"/>
+      <c r="K16" s="861"/>
+      <c r="L16" s="862"/>
       <c r="M16" s="687"/>
       <c r="O16" s="121"/>
       <c r="P16" s="682" t="s">
@@ -15134,9 +15134,9 @@
       <c r="G17" s="689"/>
       <c r="H17" s="689"/>
       <c r="I17" s="690"/>
-      <c r="J17" s="835"/>
-      <c r="K17" s="835"/>
-      <c r="L17" s="835"/>
+      <c r="J17" s="863"/>
+      <c r="K17" s="863"/>
+      <c r="L17" s="863"/>
       <c r="M17" s="691"/>
       <c r="N17" s="692"/>
       <c r="O17" s="121"/>
@@ -15159,9 +15159,9 @@
       <c r="G18" s="694"/>
       <c r="H18" s="694"/>
       <c r="I18" s="695"/>
-      <c r="J18" s="835"/>
-      <c r="K18" s="835"/>
-      <c r="L18" s="835"/>
+      <c r="J18" s="863"/>
+      <c r="K18" s="863"/>
+      <c r="L18" s="863"/>
       <c r="M18" s="691"/>
       <c r="N18" s="692"/>
       <c r="O18" s="121"/>
@@ -15181,9 +15181,9 @@
       <c r="G19" s="689"/>
       <c r="H19" s="689"/>
       <c r="I19" s="690"/>
-      <c r="J19" s="835"/>
-      <c r="K19" s="835"/>
-      <c r="L19" s="835"/>
+      <c r="J19" s="863"/>
+      <c r="K19" s="863"/>
+      <c r="L19" s="863"/>
       <c r="M19" s="691"/>
       <c r="N19" s="692"/>
       <c r="O19" s="121"/>
@@ -15203,9 +15203,9 @@
       <c r="G20" s="697"/>
       <c r="H20" s="697"/>
       <c r="I20" s="698"/>
-      <c r="J20" s="835"/>
-      <c r="K20" s="835"/>
-      <c r="L20" s="835"/>
+      <c r="J20" s="863"/>
+      <c r="K20" s="863"/>
+      <c r="L20" s="863"/>
       <c r="M20" s="691"/>
       <c r="N20" s="692"/>
       <c r="O20" s="121"/>
@@ -15225,9 +15225,9 @@
       <c r="G21" s="689"/>
       <c r="H21" s="689"/>
       <c r="I21" s="690"/>
-      <c r="J21" s="836"/>
-      <c r="K21" s="837"/>
-      <c r="L21" s="838"/>
+      <c r="J21" s="864"/>
+      <c r="K21" s="865"/>
+      <c r="L21" s="866"/>
       <c r="M21" s="691"/>
       <c r="O21" s="121"/>
       <c r="P21" s="318"/>
@@ -15247,9 +15247,9 @@
       <c r="G22" s="697"/>
       <c r="H22" s="697"/>
       <c r="I22" s="698"/>
-      <c r="J22" s="839"/>
-      <c r="K22" s="840"/>
-      <c r="L22" s="841"/>
+      <c r="J22" s="867"/>
+      <c r="K22" s="868"/>
+      <c r="L22" s="869"/>
       <c r="M22" s="691"/>
       <c r="O22" s="121"/>
       <c r="P22" s="318"/>
@@ -15269,9 +15269,9 @@
       <c r="G23" s="689"/>
       <c r="H23" s="689"/>
       <c r="I23" s="690"/>
-      <c r="J23" s="842"/>
-      <c r="K23" s="843"/>
-      <c r="L23" s="844"/>
+      <c r="J23" s="870"/>
+      <c r="K23" s="871"/>
+      <c r="L23" s="872"/>
       <c r="M23" s="691"/>
       <c r="N23" s="692"/>
       <c r="O23" s="121"/>
@@ -15282,19 +15282,19 @@
       <c r="T23" s="317"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="845" t="s">
+      <c r="B24" s="873" t="s">
         <v>285</v>
       </c>
-      <c r="C24" s="846"/>
-      <c r="D24" s="846"/>
-      <c r="E24" s="846"/>
-      <c r="F24" s="846"/>
-      <c r="G24" s="846"/>
-      <c r="H24" s="846"/>
-      <c r="I24" s="846"/>
-      <c r="J24" s="846"/>
-      <c r="K24" s="846"/>
-      <c r="L24" s="847"/>
+      <c r="C24" s="874"/>
+      <c r="D24" s="874"/>
+      <c r="E24" s="874"/>
+      <c r="F24" s="874"/>
+      <c r="G24" s="874"/>
+      <c r="H24" s="874"/>
+      <c r="I24" s="874"/>
+      <c r="J24" s="874"/>
+      <c r="K24" s="874"/>
+      <c r="L24" s="875"/>
       <c r="M24" s="699"/>
       <c r="N24" s="692"/>
       <c r="O24" s="121"/>
@@ -15341,12 +15341,12 @@
       <c r="F26" s="705"/>
       <c r="G26" s="705"/>
       <c r="H26" s="702"/>
-      <c r="I26" s="848" t="s">
+      <c r="I26" s="876" t="s">
         <v>290</v>
       </c>
-      <c r="J26" s="848"/>
-      <c r="K26" s="848"/>
-      <c r="L26" s="849"/>
+      <c r="J26" s="876"/>
+      <c r="K26" s="876"/>
+      <c r="L26" s="877"/>
       <c r="M26" s="699"/>
       <c r="N26" s="692"/>
       <c r="O26" s="121"/>
@@ -15379,26 +15379,26 @@
       <c r="T27" s="317"/>
     </row>
     <row r="28" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="832" t="s">
+      <c r="B28" s="860" t="s">
         <v>291</v>
       </c>
-      <c r="C28" s="833"/>
-      <c r="D28" s="833"/>
-      <c r="E28" s="833"/>
-      <c r="F28" s="833"/>
-      <c r="G28" s="833"/>
-      <c r="H28" s="833"/>
-      <c r="I28" s="833"/>
-      <c r="J28" s="833"/>
-      <c r="K28" s="833"/>
-      <c r="L28" s="834"/>
+      <c r="C28" s="861"/>
+      <c r="D28" s="861"/>
+      <c r="E28" s="861"/>
+      <c r="F28" s="861"/>
+      <c r="G28" s="861"/>
+      <c r="H28" s="861"/>
+      <c r="I28" s="861"/>
+      <c r="J28" s="861"/>
+      <c r="K28" s="861"/>
+      <c r="L28" s="862"/>
       <c r="M28" s="709"/>
       <c r="N28" s="692"/>
-      <c r="O28" s="831" t="s">
+      <c r="O28" s="832" t="s">
         <v>35</v>
       </c>
-      <c r="P28" s="831"/>
-      <c r="Q28" s="831"/>
+      <c r="P28" s="832"/>
+      <c r="Q28" s="832"/>
       <c r="R28" s="317"/>
       <c r="S28" s="317"/>
       <c r="T28" s="317"/>
@@ -15414,9 +15414,9 @@
       <c r="G29" s="713"/>
       <c r="H29" s="713"/>
       <c r="I29" s="714"/>
-      <c r="J29" s="850"/>
+      <c r="J29" s="830"/>
       <c r="K29" s="854"/>
-      <c r="L29" s="851"/>
+      <c r="L29" s="831"/>
       <c r="M29" s="709"/>
       <c r="N29" s="692"/>
       <c r="O29" s="716" t="s">
@@ -15476,7 +15476,7 @@
       <c r="I31" s="714"/>
       <c r="J31" s="858"/>
       <c r="K31" s="854"/>
-      <c r="L31" s="851"/>
+      <c r="L31" s="831"/>
       <c r="M31" s="722"/>
       <c r="N31" s="692"/>
       <c r="O31" s="721" t="e">
@@ -15506,9 +15506,9 @@
       <c r="G32" s="713"/>
       <c r="H32" s="713"/>
       <c r="I32" s="714"/>
-      <c r="J32" s="850"/>
+      <c r="J32" s="830"/>
       <c r="K32" s="854"/>
-      <c r="L32" s="851"/>
+      <c r="L32" s="831"/>
       <c r="N32" s="692"/>
       <c r="O32" s="721" t="e">
         <f>+LN(P32)</f>
@@ -15534,9 +15534,9 @@
       <c r="G33" s="727"/>
       <c r="H33" s="727"/>
       <c r="I33" s="728"/>
-      <c r="J33" s="850"/>
+      <c r="J33" s="830"/>
       <c r="K33" s="854"/>
-      <c r="L33" s="851"/>
+      <c r="L33" s="831"/>
       <c r="N33" s="692"/>
       <c r="O33" s="729"/>
       <c r="P33" s="444" t="s">
@@ -15555,36 +15555,36 @@
       <c r="O34" s="731"/>
     </row>
     <row r="35" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="860" t="s">
+      <c r="B35" s="840" t="s">
         <v>297</v>
       </c>
-      <c r="C35" s="861"/>
-      <c r="D35" s="861"/>
-      <c r="E35" s="861"/>
-      <c r="F35" s="862"/>
-      <c r="G35" s="866" t="s">
+      <c r="C35" s="841"/>
+      <c r="D35" s="841"/>
+      <c r="E35" s="841"/>
+      <c r="F35" s="842"/>
+      <c r="G35" s="846" t="s">
         <v>35</v>
       </c>
-      <c r="H35" s="866"/>
-      <c r="I35" s="866"/>
-      <c r="J35" s="867"/>
-      <c r="K35" s="868" t="s">
+      <c r="H35" s="846"/>
+      <c r="I35" s="846"/>
+      <c r="J35" s="847"/>
+      <c r="K35" s="848" t="s">
         <v>34</v>
       </c>
-      <c r="L35" s="866"/>
+      <c r="L35" s="846"/>
       <c r="M35" s="732"/>
       <c r="N35" s="692"/>
     </row>
     <row r="36" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="863"/>
-      <c r="C36" s="864"/>
-      <c r="D36" s="864"/>
-      <c r="E36" s="864"/>
-      <c r="F36" s="865"/>
-      <c r="G36" s="869">
+      <c r="B36" s="843"/>
+      <c r="C36" s="844"/>
+      <c r="D36" s="844"/>
+      <c r="E36" s="844"/>
+      <c r="F36" s="845"/>
+      <c r="G36" s="849">
         <v>1</v>
       </c>
-      <c r="H36" s="870"/>
+      <c r="H36" s="850"/>
       <c r="I36" s="734">
         <v>2</v>
       </c>
@@ -15599,11 +15599,11 @@
       </c>
       <c r="M36" s="732"/>
       <c r="N36" s="692"/>
-      <c r="O36" s="871" t="s">
+      <c r="O36" s="851" t="s">
         <v>244</v>
       </c>
-      <c r="P36" s="872"/>
-      <c r="Q36" s="873"/>
+      <c r="P36" s="852"/>
+      <c r="Q36" s="853"/>
       <c r="R36" s="729"/>
       <c r="S36" s="729"/>
     </row>
@@ -15617,8 +15617,8 @@
       <c r="D37" s="739"/>
       <c r="E37" s="739"/>
       <c r="F37" s="740"/>
-      <c r="G37" s="850"/>
-      <c r="H37" s="851"/>
+      <c r="G37" s="830"/>
+      <c r="H37" s="831"/>
       <c r="I37" s="737"/>
       <c r="J37" s="715"/>
       <c r="K37" s="741"/>
@@ -15629,11 +15629,11 @@
         <f>RSQ(Q30:Q32,O30:O32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="P37" s="852" t="e">
+      <c r="P37" s="828" t="e">
         <f>IF(O37&lt;=0.95,"NO CONFORME","CONFORME")</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Q37" s="853"/>
+      <c r="Q37" s="829"/>
       <c r="R37" s="729"/>
       <c r="S37" s="729"/>
     </row>
@@ -15647,8 +15647,8 @@
       <c r="D38" s="739"/>
       <c r="E38" s="739"/>
       <c r="F38" s="740"/>
-      <c r="G38" s="850"/>
-      <c r="H38" s="851"/>
+      <c r="G38" s="830"/>
+      <c r="H38" s="831"/>
       <c r="I38" s="737"/>
       <c r="J38" s="715"/>
       <c r="K38" s="745"/>
@@ -15670,19 +15670,19 @@
       <c r="F39" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G39" s="850"/>
-      <c r="H39" s="851"/>
+      <c r="G39" s="830"/>
+      <c r="H39" s="831"/>
       <c r="I39" s="737"/>
       <c r="J39" s="715"/>
       <c r="K39" s="741"/>
       <c r="L39" s="737"/>
       <c r="M39" s="747"/>
       <c r="N39" s="121"/>
-      <c r="O39" s="831" t="s">
+      <c r="O39" s="832" t="s">
         <v>34</v>
       </c>
-      <c r="P39" s="831"/>
-      <c r="Q39" s="831"/>
+      <c r="P39" s="832"/>
+      <c r="Q39" s="832"/>
       <c r="R39" s="729"/>
       <c r="S39" s="729"/>
     </row>
@@ -15698,8 +15698,8 @@
       <c r="F40" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G40" s="850"/>
-      <c r="H40" s="851"/>
+      <c r="G40" s="830"/>
+      <c r="H40" s="831"/>
       <c r="I40" s="737"/>
       <c r="J40" s="715"/>
       <c r="K40" s="741"/>
@@ -15736,8 +15736,8 @@
       <c r="F41" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G41" s="850"/>
-      <c r="H41" s="851"/>
+      <c r="G41" s="830"/>
+      <c r="H41" s="831"/>
       <c r="I41" s="737"/>
       <c r="J41" s="715"/>
       <c r="K41" s="741"/>
@@ -15762,21 +15762,21 @@
       <c r="F42" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G42" s="850"/>
-      <c r="H42" s="851"/>
+      <c r="G42" s="830"/>
+      <c r="H42" s="831"/>
       <c r="I42" s="737"/>
       <c r="J42" s="715"/>
       <c r="K42" s="741"/>
       <c r="L42" s="737"/>
       <c r="M42" s="747"/>
       <c r="N42" s="121"/>
-      <c r="O42" s="874" t="s">
+      <c r="O42" s="833" t="s">
         <v>217</v>
       </c>
-      <c r="P42" s="875"/>
-      <c r="Q42" s="875"/>
-      <c r="R42" s="875"/>
-      <c r="S42" s="876"/>
+      <c r="P42" s="834"/>
+      <c r="Q42" s="834"/>
+      <c r="R42" s="834"/>
+      <c r="S42" s="835"/>
     </row>
     <row r="43" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="737" t="s">
@@ -15790,11 +15790,11 @@
       <c r="F43" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G43" s="852">
+      <c r="G43" s="828">
         <f>+G39-G41</f>
         <v>0</v>
       </c>
-      <c r="H43" s="853"/>
+      <c r="H43" s="829"/>
       <c r="I43" s="743">
         <f>+I39-I41</f>
         <v>0</v>
@@ -15813,15 +15813,15 @@
       </c>
       <c r="M43" s="747"/>
       <c r="N43" s="121"/>
-      <c r="O43" s="877" t="s">
+      <c r="O43" s="836" t="s">
         <v>212</v>
       </c>
-      <c r="P43" s="878"/>
-      <c r="Q43" s="877" t="s">
+      <c r="P43" s="837"/>
+      <c r="Q43" s="836" t="s">
         <v>213</v>
       </c>
-      <c r="R43" s="878"/>
-      <c r="S43" s="879" t="s">
+      <c r="R43" s="837"/>
+      <c r="S43" s="838" t="s">
         <v>214</v>
       </c>
     </row>
@@ -15837,11 +15837,11 @@
       <c r="F44" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G44" s="850">
+      <c r="G44" s="830">
         <f>+G41-G42</f>
         <v>0</v>
       </c>
-      <c r="H44" s="851"/>
+      <c r="H44" s="831"/>
       <c r="I44" s="737">
         <f>+I41-I42</f>
         <v>0</v>
@@ -15872,7 +15872,7 @@
       <c r="R44" s="750" t="s">
         <v>216</v>
       </c>
-      <c r="S44" s="880"/>
+      <c r="S44" s="839"/>
     </row>
     <row r="45" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="737" t="s">
@@ -15886,11 +15886,11 @@
       <c r="F45" s="736" t="s">
         <v>110</v>
       </c>
-      <c r="G45" s="852" t="e">
+      <c r="G45" s="828" t="e">
         <f>+G43/G44*100</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H45" s="853"/>
+      <c r="H45" s="829"/>
       <c r="I45" s="743" t="e">
         <f>+I43/I44*100</f>
         <v>#DIV/0!</v>
@@ -15943,15 +15943,15 @@
     </row>
     <row r="47" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="753"/>
-      <c r="B47" s="883" t="s">
+      <c r="B47" s="822" t="s">
         <v>308</v>
       </c>
-      <c r="C47" s="884"/>
-      <c r="D47" s="883" t="s">
+      <c r="C47" s="823"/>
+      <c r="D47" s="822" t="s">
         <v>309</v>
       </c>
-      <c r="E47" s="885"/>
-      <c r="F47" s="884"/>
+      <c r="E47" s="824"/>
+      <c r="F47" s="823"/>
       <c r="G47" s="754" t="s">
         <v>310</v>
       </c>
@@ -15967,9 +15967,9 @@
         <v>311</v>
       </c>
       <c r="C48" s="759"/>
-      <c r="D48" s="886"/>
-      <c r="E48" s="887"/>
-      <c r="F48" s="888"/>
+      <c r="D48" s="825"/>
+      <c r="E48" s="826"/>
+      <c r="F48" s="827"/>
       <c r="G48" s="760"/>
       <c r="H48" s="725"/>
       <c r="I48" s="725"/>
@@ -15983,9 +15983,9 @@
         <v>312</v>
       </c>
       <c r="C49" s="759"/>
-      <c r="D49" s="886"/>
-      <c r="E49" s="887"/>
-      <c r="F49" s="888"/>
+      <c r="D49" s="825"/>
+      <c r="E49" s="826"/>
+      <c r="F49" s="827"/>
       <c r="G49" s="762"/>
       <c r="N49" s="121"/>
     </row>
@@ -15994,9 +15994,9 @@
         <v>313</v>
       </c>
       <c r="C50" s="759"/>
-      <c r="D50" s="886"/>
-      <c r="E50" s="887"/>
-      <c r="F50" s="888"/>
+      <c r="D50" s="825"/>
+      <c r="E50" s="826"/>
+      <c r="F50" s="827"/>
       <c r="N50" s="121"/>
     </row>
     <row r="51" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -16004,17 +16004,17 @@
         <v>314</v>
       </c>
       <c r="C51" s="759"/>
-      <c r="D51" s="886"/>
-      <c r="E51" s="887"/>
-      <c r="F51" s="888"/>
+      <c r="D51" s="825"/>
+      <c r="E51" s="826"/>
+      <c r="F51" s="827"/>
       <c r="N51" s="121"/>
     </row>
     <row r="52" spans="1:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="763"/>
       <c r="C52" s="764"/>
-      <c r="D52" s="881"/>
-      <c r="E52" s="881"/>
-      <c r="F52" s="881"/>
+      <c r="D52" s="820"/>
+      <c r="E52" s="820"/>
+      <c r="F52" s="820"/>
       <c r="N52" s="121"/>
       <c r="O52" s="121"/>
     </row>
@@ -16060,21 +16060,21 @@
     </row>
     <row r="55" spans="1:15" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="882" t="s">
+      <c r="A56" s="821" t="s">
         <v>318</v>
       </c>
-      <c r="B56" s="882"/>
-      <c r="C56" s="882"/>
-      <c r="D56" s="882"/>
-      <c r="E56" s="882"/>
-      <c r="F56" s="882"/>
-      <c r="G56" s="882"/>
-      <c r="H56" s="882"/>
-      <c r="I56" s="882"/>
-      <c r="J56" s="882"/>
-      <c r="K56" s="882"/>
-      <c r="L56" s="882"/>
-      <c r="M56" s="882"/>
+      <c r="B56" s="821"/>
+      <c r="C56" s="821"/>
+      <c r="D56" s="821"/>
+      <c r="E56" s="821"/>
+      <c r="F56" s="821"/>
+      <c r="G56" s="821"/>
+      <c r="H56" s="821"/>
+      <c r="I56" s="821"/>
+      <c r="J56" s="821"/>
+      <c r="K56" s="821"/>
+      <c r="L56" s="821"/>
+      <c r="M56" s="821"/>
     </row>
     <row r="57" spans="1:15" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:15" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16085,14 +16085,43 @@
     <protectedRange sqref="C10:E11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="58">
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="A56:M56"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="A13:M13"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="I26:L26"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="P37:Q37"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="J32:L32"/>
+    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="B35:F36"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="O36:Q36"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="G38:H38"/>
     <mergeCell ref="G39:H39"/>
@@ -16106,43 +16135,14 @@
     <mergeCell ref="Q43:R43"/>
     <mergeCell ref="S43:S44"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="B35:F36"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="O36:Q36"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="P37:Q37"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="J32:L32"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="B16:L16"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="B24:L24"/>
-    <mergeCell ref="I26:L26"/>
-    <mergeCell ref="B28:L28"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A7:M7"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="A13:M13"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A56:M56"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="D51:F51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16194,43 +16194,43 @@
       <c r="N1" s="205"/>
     </row>
     <row r="2" spans="1:36" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="790" t="s">
+      <c r="A2" s="802" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="790"/>
-      <c r="C2" s="790"/>
-      <c r="D2" s="790"/>
-      <c r="E2" s="790"/>
-      <c r="F2" s="790"/>
-      <c r="G2" s="790"/>
-      <c r="H2" s="790"/>
-      <c r="I2" s="790"/>
-      <c r="J2" s="790"/>
-      <c r="K2" s="790"/>
-      <c r="L2" s="790"/>
-      <c r="M2" s="790"/>
-      <c r="N2" s="790"/>
+      <c r="B2" s="802"/>
+      <c r="C2" s="802"/>
+      <c r="D2" s="802"/>
+      <c r="E2" s="802"/>
+      <c r="F2" s="802"/>
+      <c r="G2" s="802"/>
+      <c r="H2" s="802"/>
+      <c r="I2" s="802"/>
+      <c r="J2" s="802"/>
+      <c r="K2" s="802"/>
+      <c r="L2" s="802"/>
+      <c r="M2" s="802"/>
+      <c r="N2" s="802"/>
       <c r="AJ2" s="180" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:36" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="899">
-        <v>0</v>
-      </c>
-      <c r="B3" s="899"/>
-      <c r="C3" s="899"/>
-      <c r="D3" s="899"/>
-      <c r="E3" s="899"/>
-      <c r="F3" s="899"/>
-      <c r="G3" s="899"/>
-      <c r="H3" s="899"/>
-      <c r="I3" s="899"/>
-      <c r="J3" s="899"/>
-      <c r="K3" s="899"/>
-      <c r="L3" s="899"/>
-      <c r="M3" s="899"/>
-      <c r="N3" s="899"/>
+      <c r="A3" s="902">
+        <v>0</v>
+      </c>
+      <c r="B3" s="902"/>
+      <c r="C3" s="902"/>
+      <c r="D3" s="902"/>
+      <c r="E3" s="902"/>
+      <c r="F3" s="902"/>
+      <c r="G3" s="902"/>
+      <c r="H3" s="902"/>
+      <c r="I3" s="902"/>
+      <c r="J3" s="902"/>
+      <c r="K3" s="902"/>
+      <c r="L3" s="902"/>
+      <c r="M3" s="902"/>
+      <c r="N3" s="902"/>
       <c r="AJ3" s="180" t="s">
         <v>145</v>
       </c>
@@ -16249,18 +16249,18 @@
       <c r="B5" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="903">
+      <c r="C5" s="906">
         <f>+FORMATO!Q2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="903"/>
-      <c r="E5" s="903"/>
-      <c r="F5" s="903"/>
-      <c r="G5" s="903"/>
-      <c r="H5" s="903"/>
-      <c r="I5" s="903"/>
-      <c r="J5" s="903"/>
-      <c r="K5" s="903"/>
+      <c r="D5" s="906"/>
+      <c r="E5" s="906"/>
+      <c r="F5" s="906"/>
+      <c r="G5" s="906"/>
+      <c r="H5" s="906"/>
+      <c r="I5" s="906"/>
+      <c r="J5" s="906"/>
+      <c r="K5" s="906"/>
       <c r="L5" s="30" t="s">
         <v>21</v>
       </c>
@@ -16278,17 +16278,17 @@
       <c r="B6" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="902">
+      <c r="C6" s="905">
         <f>+FORMATO!Q3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="902"/>
-      <c r="E6" s="902"/>
-      <c r="F6" s="902"/>
-      <c r="G6" s="902"/>
-      <c r="H6" s="902"/>
-      <c r="I6" s="902"/>
-      <c r="J6" s="902"/>
+      <c r="D6" s="905"/>
+      <c r="E6" s="905"/>
+      <c r="F6" s="905"/>
+      <c r="G6" s="905"/>
+      <c r="H6" s="905"/>
+      <c r="I6" s="905"/>
+      <c r="J6" s="905"/>
       <c r="K6" s="40"/>
       <c r="L6" s="34" t="s">
         <v>269</v>
@@ -16316,18 +16316,18 @@
       <c r="B7" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="903">
+      <c r="C7" s="906">
         <f>+FORMATO!Q4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="903"/>
-      <c r="E7" s="903"/>
-      <c r="F7" s="903"/>
-      <c r="G7" s="903"/>
-      <c r="H7" s="903"/>
-      <c r="I7" s="903"/>
-      <c r="J7" s="903"/>
-      <c r="K7" s="903"/>
+      <c r="D7" s="906"/>
+      <c r="E7" s="906"/>
+      <c r="F7" s="906"/>
+      <c r="G7" s="906"/>
+      <c r="H7" s="906"/>
+      <c r="I7" s="906"/>
+      <c r="J7" s="906"/>
+      <c r="K7" s="906"/>
       <c r="L7" s="34" t="s">
         <v>320</v>
       </c>
@@ -16359,17 +16359,17 @@
       <c r="B8" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="902">
+      <c r="C8" s="905">
         <f>+FORMATO!Q5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="902"/>
-      <c r="E8" s="902"/>
-      <c r="F8" s="902"/>
-      <c r="G8" s="902"/>
-      <c r="H8" s="902"/>
-      <c r="I8" s="902"/>
-      <c r="J8" s="902"/>
+      <c r="D8" s="905"/>
+      <c r="E8" s="905"/>
+      <c r="F8" s="905"/>
+      <c r="G8" s="905"/>
+      <c r="H8" s="905"/>
+      <c r="I8" s="905"/>
+      <c r="J8" s="905"/>
       <c r="K8" s="780"/>
       <c r="L8" s="34" t="s">
         <v>115</v>
@@ -16391,9 +16391,9 @@
       <c r="Y8" s="185"/>
       <c r="Z8" s="185"/>
       <c r="AA8" s="185"/>
-      <c r="AB8" s="890"/>
-      <c r="AC8" s="890"/>
-      <c r="AD8" s="890"/>
+      <c r="AB8" s="907"/>
+      <c r="AC8" s="907"/>
+      <c r="AD8" s="907"/>
     </row>
     <row r="9" spans="1:36" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="629" t="s">
@@ -16427,22 +16427,22 @@
       <c r="AD9" s="244"/>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A10" s="891" t="s">
+      <c r="A10" s="908" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="892"/>
-      <c r="C10" s="892"/>
-      <c r="D10" s="892"/>
-      <c r="E10" s="892"/>
-      <c r="F10" s="892"/>
-      <c r="G10" s="892"/>
-      <c r="H10" s="892"/>
-      <c r="I10" s="892"/>
-      <c r="J10" s="892"/>
-      <c r="K10" s="892"/>
-      <c r="L10" s="892"/>
-      <c r="M10" s="892"/>
-      <c r="N10" s="893"/>
+      <c r="B10" s="909"/>
+      <c r="C10" s="909"/>
+      <c r="D10" s="909"/>
+      <c r="E10" s="909"/>
+      <c r="F10" s="909"/>
+      <c r="G10" s="909"/>
+      <c r="H10" s="909"/>
+      <c r="I10" s="909"/>
+      <c r="J10" s="909"/>
+      <c r="K10" s="909"/>
+      <c r="L10" s="909"/>
+      <c r="M10" s="909"/>
+      <c r="N10" s="910"/>
       <c r="O10" s="183"/>
       <c r="P10" s="183"/>
       <c r="Q10" s="183"/>
@@ -16458,22 +16458,22 @@
       <c r="AD10" s="244"/>
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A11" s="894" t="s">
+      <c r="A11" s="911" t="s">
         <v>236</v>
       </c>
-      <c r="B11" s="895"/>
-      <c r="C11" s="895"/>
-      <c r="D11" s="895"/>
-      <c r="E11" s="895"/>
-      <c r="F11" s="895"/>
-      <c r="G11" s="895"/>
-      <c r="H11" s="895"/>
-      <c r="I11" s="895"/>
-      <c r="J11" s="895"/>
-      <c r="K11" s="895"/>
-      <c r="L11" s="895"/>
-      <c r="M11" s="895"/>
-      <c r="N11" s="896"/>
+      <c r="B11" s="912"/>
+      <c r="C11" s="912"/>
+      <c r="D11" s="912"/>
+      <c r="E11" s="912"/>
+      <c r="F11" s="912"/>
+      <c r="G11" s="912"/>
+      <c r="H11" s="912"/>
+      <c r="I11" s="912"/>
+      <c r="J11" s="912"/>
+      <c r="K11" s="912"/>
+      <c r="L11" s="912"/>
+      <c r="M11" s="912"/>
+      <c r="N11" s="913"/>
       <c r="O11" s="183"/>
       <c r="P11" s="183"/>
       <c r="Q11" s="183"/>
@@ -16750,8 +16750,8 @@
       <c r="I19" s="211"/>
       <c r="J19" s="211"/>
       <c r="K19" s="211"/>
-      <c r="L19" s="791"/>
-      <c r="M19" s="791"/>
+      <c r="L19" s="803"/>
+      <c r="M19" s="803"/>
       <c r="N19" s="53"/>
       <c r="O19" s="183"/>
       <c r="P19" s="198"/>
@@ -16759,18 +16759,18 @@
       <c r="R19" s="198"/>
       <c r="S19" s="198"/>
       <c r="T19" s="198"/>
-      <c r="U19" s="889" t="s">
+      <c r="U19" s="890" t="s">
         <v>197</v>
       </c>
-      <c r="V19" s="898" t="s">
+      <c r="V19" s="915" t="s">
         <v>35</v>
       </c>
-      <c r="W19" s="898"/>
-      <c r="X19" s="898"/>
-      <c r="Y19" s="898" t="s">
+      <c r="W19" s="915"/>
+      <c r="X19" s="915"/>
+      <c r="Y19" s="915" t="s">
         <v>34</v>
       </c>
-      <c r="Z19" s="898"/>
+      <c r="Z19" s="915"/>
       <c r="AA19" s="199"/>
       <c r="AB19" s="199"/>
       <c r="AC19" s="199"/>
@@ -16779,27 +16779,27 @@
       <c r="AF19" s="199"/>
     </row>
     <row r="20" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="793" t="s">
+      <c r="A20" s="805" t="s">
         <v>146</v>
       </c>
-      <c r="B20" s="794"/>
-      <c r="C20" s="794"/>
-      <c r="D20" s="794"/>
-      <c r="E20" s="794"/>
+      <c r="B20" s="806"/>
+      <c r="C20" s="806"/>
+      <c r="D20" s="806"/>
+      <c r="E20" s="806"/>
       <c r="F20" s="212" t="s">
         <v>113</v>
       </c>
-      <c r="G20" s="793" t="s">
+      <c r="G20" s="805" t="s">
         <v>206</v>
       </c>
-      <c r="H20" s="794"/>
-      <c r="I20" s="900"/>
-      <c r="J20" s="901" t="s">
+      <c r="H20" s="806"/>
+      <c r="I20" s="903"/>
+      <c r="J20" s="904" t="s">
         <v>205</v>
       </c>
-      <c r="K20" s="796"/>
-      <c r="L20" s="792"/>
-      <c r="M20" s="792"/>
+      <c r="K20" s="808"/>
+      <c r="L20" s="804"/>
+      <c r="M20" s="804"/>
       <c r="N20" s="57"/>
       <c r="O20" s="183"/>
       <c r="P20" s="200"/>
@@ -16807,18 +16807,18 @@
       <c r="R20" s="200"/>
       <c r="S20" s="200"/>
       <c r="T20" s="200"/>
-      <c r="U20" s="889"/>
-      <c r="V20" s="897" t="str">
+      <c r="U20" s="890"/>
+      <c r="V20" s="914" t="str">
         <f>+DATOS!C12</f>
         <v>-</v>
       </c>
-      <c r="W20" s="897"/>
-      <c r="X20" s="897"/>
-      <c r="Y20" s="897" t="str">
+      <c r="W20" s="914"/>
+      <c r="X20" s="914"/>
+      <c r="Y20" s="914" t="str">
         <f>+DATOS!I12</f>
         <v>-</v>
       </c>
-      <c r="Z20" s="897"/>
+      <c r="Z20" s="914"/>
       <c r="AA20" s="199"/>
       <c r="AB20" s="199"/>
       <c r="AC20" s="199"/>
@@ -16827,13 +16827,13 @@
       <c r="AF20" s="199"/>
     </row>
     <row r="21" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="808" t="s">
+      <c r="A21" s="793" t="s">
         <v>147</v>
       </c>
-      <c r="B21" s="809"/>
-      <c r="C21" s="809"/>
-      <c r="D21" s="809"/>
-      <c r="E21" s="810"/>
+      <c r="B21" s="794"/>
+      <c r="C21" s="794"/>
+      <c r="D21" s="794"/>
+      <c r="E21" s="795"/>
       <c r="F21" s="213" t="s">
         <v>148</v>
       </c>
@@ -16857,8 +16857,8 @@
         <f>IF($Y$20="NO",Z21,IF($Y$20="-","",Z21))</f>
         <v/>
       </c>
-      <c r="L21" s="792"/>
-      <c r="M21" s="792"/>
+      <c r="L21" s="804"/>
+      <c r="M21" s="804"/>
       <c r="N21" s="57"/>
       <c r="O21" s="183"/>
       <c r="P21" s="200"/>
@@ -16892,13 +16892,13 @@
       <c r="AF21" s="199"/>
     </row>
     <row r="22" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="787" t="s">
+      <c r="A22" s="790" t="s">
         <v>149</v>
       </c>
-      <c r="B22" s="788"/>
-      <c r="C22" s="788"/>
-      <c r="D22" s="788"/>
-      <c r="E22" s="789"/>
+      <c r="B22" s="791"/>
+      <c r="C22" s="791"/>
+      <c r="D22" s="791"/>
+      <c r="E22" s="792"/>
       <c r="F22" s="213" t="s">
         <v>148</v>
       </c>
@@ -16922,8 +16922,8 @@
         <f>IF($Y$20="NO","--",IF($Y$20="-","",Z22))</f>
         <v/>
       </c>
-      <c r="L22" s="801"/>
-      <c r="M22" s="801"/>
+      <c r="L22" s="813"/>
+      <c r="M22" s="813"/>
       <c r="N22" s="69"/>
       <c r="O22" s="201"/>
       <c r="P22" s="200"/>
@@ -16962,13 +16962,13 @@
       <c r="AF22" s="199"/>
     </row>
     <row r="23" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="787" t="s">
+      <c r="A23" s="790" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="788"/>
-      <c r="C23" s="788"/>
-      <c r="D23" s="788"/>
-      <c r="E23" s="789"/>
+      <c r="B23" s="791"/>
+      <c r="C23" s="791"/>
+      <c r="D23" s="791"/>
+      <c r="E23" s="792"/>
       <c r="F23" s="213" t="s">
         <v>148</v>
       </c>
@@ -17024,13 +17024,13 @@
       <c r="AF23" s="199"/>
     </row>
     <row r="24" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="787" t="s">
+      <c r="A24" s="790" t="s">
         <v>208</v>
       </c>
-      <c r="B24" s="788"/>
-      <c r="C24" s="788"/>
-      <c r="D24" s="788"/>
-      <c r="E24" s="789"/>
+      <c r="B24" s="791"/>
+      <c r="C24" s="791"/>
+      <c r="D24" s="791"/>
+      <c r="E24" s="792"/>
       <c r="F24" s="213" t="s">
         <v>109</v>
       </c>
@@ -17094,13 +17094,13 @@
       <c r="AF24" s="199"/>
     </row>
     <row r="25" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="787" t="s">
+      <c r="A25" s="790" t="s">
         <v>209</v>
       </c>
-      <c r="B25" s="788"/>
-      <c r="C25" s="788"/>
-      <c r="D25" s="788"/>
-      <c r="E25" s="789"/>
+      <c r="B25" s="791"/>
+      <c r="C25" s="791"/>
+      <c r="D25" s="791"/>
+      <c r="E25" s="792"/>
       <c r="F25" s="213" t="s">
         <v>109</v>
       </c>
@@ -17164,13 +17164,13 @@
       <c r="AF25" s="199"/>
     </row>
     <row r="26" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="787" t="s">
+      <c r="A26" s="790" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="788"/>
-      <c r="C26" s="788"/>
-      <c r="D26" s="788"/>
-      <c r="E26" s="789"/>
+      <c r="B26" s="791"/>
+      <c r="C26" s="791"/>
+      <c r="D26" s="791"/>
+      <c r="E26" s="792"/>
       <c r="F26" s="213" t="s">
         <v>109</v>
       </c>
@@ -17234,13 +17234,13 @@
       <c r="AF26" s="199"/>
     </row>
     <row r="27" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="787" t="s">
+      <c r="A27" s="790" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="788"/>
-      <c r="C27" s="788"/>
-      <c r="D27" s="788"/>
-      <c r="E27" s="789"/>
+      <c r="B27" s="791"/>
+      <c r="C27" s="791"/>
+      <c r="D27" s="791"/>
+      <c r="E27" s="792"/>
       <c r="F27" s="213" t="s">
         <v>109</v>
       </c>
@@ -17304,13 +17304,13 @@
       <c r="AF27" s="199"/>
     </row>
     <row r="28" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="787" t="s">
+      <c r="A28" s="790" t="s">
         <v>210</v>
       </c>
-      <c r="B28" s="788"/>
-      <c r="C28" s="788"/>
-      <c r="D28" s="788"/>
-      <c r="E28" s="789"/>
+      <c r="B28" s="791"/>
+      <c r="C28" s="791"/>
+      <c r="D28" s="791"/>
+      <c r="E28" s="792"/>
       <c r="F28" s="213" t="s">
         <v>109</v>
       </c>
@@ -17374,13 +17374,13 @@
       <c r="AF28" s="199"/>
     </row>
     <row r="29" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="808" t="s">
+      <c r="A29" s="793" t="s">
         <v>111</v>
       </c>
-      <c r="B29" s="809"/>
-      <c r="C29" s="809"/>
-      <c r="D29" s="809"/>
-      <c r="E29" s="810"/>
+      <c r="B29" s="794"/>
+      <c r="C29" s="794"/>
+      <c r="D29" s="794"/>
+      <c r="E29" s="795"/>
       <c r="F29" s="217" t="s">
         <v>110</v>
       </c>
@@ -17521,11 +17521,11 @@
       <c r="V31" s="180"/>
       <c r="W31" s="233"/>
       <c r="X31" s="261"/>
-      <c r="Y31" s="904" t="e">
+      <c r="Y31" s="901" t="e">
         <f>AVERAGE(Y30:Z30)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z31" s="904"/>
+      <c r="Z31" s="901"/>
       <c r="AA31" s="199"/>
       <c r="AB31" s="199"/>
       <c r="AC31" s="199"/>
@@ -17543,10 +17543,10 @@
       <c r="G32" s="21"/>
       <c r="H32" s="21"/>
       <c r="I32" s="21"/>
-      <c r="J32" s="811" t="s">
+      <c r="J32" s="781" t="s">
         <v>203</v>
       </c>
-      <c r="K32" s="812"/>
+      <c r="K32" s="782"/>
       <c r="L32" s="221" t="str">
         <f>IF(V20="-","",IF(V20="NO","NP",ROUND(V42,0)))</f>
         <v/>
@@ -17620,10 +17620,10 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
       <c r="I34" s="21"/>
-      <c r="J34" s="811" t="s">
+      <c r="J34" s="781" t="s">
         <v>204</v>
       </c>
-      <c r="K34" s="812"/>
+      <c r="K34" s="782"/>
       <c r="L34" s="221" t="str">
         <f>IF(V20="-","",IF(Y20="NO","NP",ROUND(Y31,0)))</f>
         <v/>
@@ -17717,10 +17717,10 @@
       <c r="G36" s="209"/>
       <c r="H36" s="209"/>
       <c r="I36" s="209"/>
-      <c r="J36" s="811" t="s">
+      <c r="J36" s="781" t="s">
         <v>77</v>
       </c>
-      <c r="K36" s="812"/>
+      <c r="K36" s="782"/>
       <c r="L36" s="221" t="str">
         <f>IF(Y20="-","",IF(Y20="NO","NP",L32-L34))</f>
         <v/>
@@ -17970,10 +17970,10 @@
       </c>
       <c r="V42" s="598"/>
       <c r="W42" s="525"/>
-      <c r="X42" s="905" t="s">
+      <c r="X42" s="892" t="s">
         <v>175</v>
       </c>
-      <c r="Y42" s="906"/>
+      <c r="Y42" s="893"/>
       <c r="Z42" s="577" t="e">
         <f>(Z39*LN(25)+Z40)</f>
         <v>#VALUE!</v>
@@ -18263,13 +18263,13 @@
       <c r="H52" s="293"/>
       <c r="I52" s="231"/>
       <c r="J52" s="231"/>
-      <c r="K52" s="889">
+      <c r="K52" s="890">
         <f>+FORMATO!J17</f>
         <v>0</v>
       </c>
-      <c r="L52" s="889"/>
-      <c r="M52" s="889"/>
-      <c r="N52" s="889"/>
+      <c r="L52" s="890"/>
+      <c r="M52" s="890"/>
+      <c r="N52" s="890"/>
       <c r="O52" s="203"/>
       <c r="P52" s="183"/>
       <c r="Q52" s="183"/>
@@ -18290,13 +18290,13 @@
       <c r="H53" s="293"/>
       <c r="I53" s="231"/>
       <c r="J53" s="231"/>
-      <c r="K53" s="889">
+      <c r="K53" s="890">
         <f>+FORMATO!J18</f>
         <v>0</v>
       </c>
-      <c r="L53" s="889"/>
-      <c r="M53" s="889"/>
-      <c r="N53" s="889"/>
+      <c r="L53" s="890"/>
+      <c r="M53" s="890"/>
+      <c r="N53" s="890"/>
       <c r="O53" s="203"/>
       <c r="P53" s="183"/>
       <c r="Q53" s="183"/>
@@ -18317,13 +18317,13 @@
       <c r="H54" s="293"/>
       <c r="I54" s="231"/>
       <c r="J54" s="231"/>
-      <c r="K54" s="889">
+      <c r="K54" s="890">
         <f>+FORMATO!J19</f>
         <v>0</v>
       </c>
-      <c r="L54" s="889"/>
-      <c r="M54" s="889"/>
-      <c r="N54" s="889"/>
+      <c r="L54" s="890"/>
+      <c r="M54" s="890"/>
+      <c r="N54" s="890"/>
       <c r="O54" s="203"/>
       <c r="P54" s="183"/>
       <c r="Q54" s="183"/>
@@ -18344,13 +18344,13 @@
       <c r="H55" s="293"/>
       <c r="I55" s="231"/>
       <c r="J55" s="231"/>
-      <c r="K55" s="889">
+      <c r="K55" s="890">
         <f>+FORMATO!J20</f>
         <v>0</v>
       </c>
-      <c r="L55" s="889"/>
-      <c r="M55" s="889"/>
-      <c r="N55" s="889"/>
+      <c r="L55" s="890"/>
+      <c r="M55" s="890"/>
+      <c r="N55" s="890"/>
       <c r="O55" s="203"/>
       <c r="P55" s="183"/>
       <c r="Q55" s="183"/>
@@ -18372,13 +18372,13 @@
       <c r="H56" s="293"/>
       <c r="I56" s="231"/>
       <c r="J56" s="231"/>
-      <c r="K56" s="889">
+      <c r="K56" s="890">
         <f>+FORMATO!J22</f>
         <v>0</v>
       </c>
-      <c r="L56" s="889"/>
-      <c r="M56" s="889"/>
-      <c r="N56" s="889"/>
+      <c r="L56" s="890"/>
+      <c r="M56" s="890"/>
+      <c r="N56" s="890"/>
       <c r="O56" s="203"/>
       <c r="P56" s="183"/>
       <c r="Q56" s="183"/>
@@ -18399,13 +18399,13 @@
       <c r="H57" s="231"/>
       <c r="I57" s="231"/>
       <c r="J57" s="231"/>
-      <c r="K57" s="889">
+      <c r="K57" s="890">
         <f>+FORMATO!J23</f>
         <v>0</v>
       </c>
-      <c r="L57" s="889"/>
-      <c r="M57" s="889"/>
-      <c r="N57" s="889"/>
+      <c r="L57" s="890"/>
+      <c r="M57" s="890"/>
+      <c r="N57" s="890"/>
       <c r="O57" s="290"/>
       <c r="P57" s="183"/>
       <c r="Q57" s="183"/>
@@ -18469,11 +18469,11 @@
       <c r="F60" s="179"/>
       <c r="G60" s="179"/>
       <c r="H60" s="179"/>
-      <c r="I60" s="889">
+      <c r="I60" s="890">
         <f>+FORMATO!J29</f>
         <v>0</v>
       </c>
-      <c r="J60" s="889"/>
+      <c r="J60" s="890"/>
       <c r="K60" s="231"/>
       <c r="L60" s="231"/>
       <c r="M60" s="231"/>
@@ -18495,11 +18495,11 @@
       <c r="F61" s="179"/>
       <c r="G61" s="179"/>
       <c r="H61" s="179"/>
-      <c r="I61" s="889">
+      <c r="I61" s="890">
         <f>+FORMATO!J30</f>
         <v>0</v>
       </c>
-      <c r="J61" s="889"/>
+      <c r="J61" s="890"/>
       <c r="K61" s="231"/>
       <c r="L61" s="231"/>
       <c r="M61" s="231"/>
@@ -18521,11 +18521,11 @@
       <c r="F62" s="179"/>
       <c r="G62" s="179"/>
       <c r="H62" s="179"/>
-      <c r="I62" s="889">
+      <c r="I62" s="890">
         <f>+FORMATO!J31</f>
         <v>0</v>
       </c>
-      <c r="J62" s="889"/>
+      <c r="J62" s="890"/>
       <c r="K62" s="231"/>
       <c r="L62" s="231"/>
       <c r="M62" s="231"/>
@@ -18547,11 +18547,11 @@
       <c r="F63" s="179"/>
       <c r="G63" s="179"/>
       <c r="H63" s="179"/>
-      <c r="I63" s="909">
+      <c r="I63" s="895">
         <f>+FORMATO!J32</f>
         <v>0</v>
       </c>
-      <c r="J63" s="909"/>
+      <c r="J63" s="895"/>
       <c r="K63" s="231"/>
       <c r="L63" s="231"/>
       <c r="M63" s="231"/>
@@ -18573,11 +18573,11 @@
       <c r="F64" s="179"/>
       <c r="G64" s="179"/>
       <c r="H64" s="179"/>
-      <c r="I64" s="889">
+      <c r="I64" s="890">
         <f>+FORMATO!J33</f>
         <v>0</v>
       </c>
-      <c r="J64" s="889"/>
+      <c r="J64" s="890"/>
       <c r="K64" s="231"/>
       <c r="L64" s="231"/>
       <c r="M64" s="231"/>
@@ -18599,17 +18599,17 @@
       <c r="F65" s="301"/>
       <c r="G65" s="301"/>
       <c r="H65" s="301"/>
-      <c r="I65" s="910">
+      <c r="I65" s="896">
         <f>+FORMATO!J21</f>
         <v>0</v>
       </c>
-      <c r="J65" s="910"/>
-      <c r="K65" s="912">
-        <v>0</v>
-      </c>
-      <c r="L65" s="913"/>
-      <c r="M65" s="913"/>
-      <c r="N65" s="913"/>
+      <c r="J65" s="896"/>
+      <c r="K65" s="898">
+        <v>0</v>
+      </c>
+      <c r="L65" s="899"/>
+      <c r="M65" s="899"/>
+      <c r="N65" s="899"/>
       <c r="O65" s="296"/>
       <c r="P65" s="183"/>
       <c r="Q65" s="179"/>
@@ -18652,94 +18652,94 @@
       <c r="N67" s="178"/>
     </row>
     <row r="68" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="914" t="s">
+      <c r="A68" s="900" t="s">
         <v>337</v>
       </c>
-      <c r="B68" s="914"/>
-      <c r="C68" s="914"/>
-      <c r="D68" s="914"/>
-      <c r="E68" s="914"/>
-      <c r="F68" s="914"/>
-      <c r="G68" s="914"/>
-      <c r="H68" s="914"/>
-      <c r="I68" s="914"/>
-      <c r="J68" s="914"/>
-      <c r="K68" s="914"/>
-      <c r="L68" s="914"/>
-      <c r="M68" s="914"/>
-      <c r="N68" s="914"/>
+      <c r="B68" s="900"/>
+      <c r="C68" s="900"/>
+      <c r="D68" s="900"/>
+      <c r="E68" s="900"/>
+      <c r="F68" s="900"/>
+      <c r="G68" s="900"/>
+      <c r="H68" s="900"/>
+      <c r="I68" s="900"/>
+      <c r="J68" s="900"/>
+      <c r="K68" s="900"/>
+      <c r="L68" s="900"/>
+      <c r="M68" s="900"/>
+      <c r="N68" s="900"/>
     </row>
     <row r="69" spans="1:19" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="911" t="s">
+      <c r="A69" s="897" t="s">
         <v>338</v>
       </c>
-      <c r="B69" s="911"/>
-      <c r="C69" s="911"/>
-      <c r="D69" s="911"/>
-      <c r="E69" s="911"/>
-      <c r="F69" s="911"/>
-      <c r="G69" s="911"/>
-      <c r="H69" s="911"/>
-      <c r="I69" s="911"/>
-      <c r="J69" s="911"/>
-      <c r="K69" s="911"/>
-      <c r="L69" s="911"/>
-      <c r="M69" s="911"/>
-      <c r="N69" s="911"/>
+      <c r="B69" s="897"/>
+      <c r="C69" s="897"/>
+      <c r="D69" s="897"/>
+      <c r="E69" s="897"/>
+      <c r="F69" s="897"/>
+      <c r="G69" s="897"/>
+      <c r="H69" s="897"/>
+      <c r="I69" s="897"/>
+      <c r="J69" s="897"/>
+      <c r="K69" s="897"/>
+      <c r="L69" s="897"/>
+      <c r="M69" s="897"/>
+      <c r="N69" s="897"/>
     </row>
     <row r="70" spans="1:19" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="911" t="s">
+      <c r="A70" s="897" t="s">
         <v>339</v>
       </c>
-      <c r="B70" s="911"/>
-      <c r="C70" s="911"/>
-      <c r="D70" s="911"/>
-      <c r="E70" s="911"/>
-      <c r="F70" s="911"/>
-      <c r="G70" s="911"/>
-      <c r="H70" s="911"/>
-      <c r="I70" s="911"/>
-      <c r="J70" s="911"/>
-      <c r="K70" s="911"/>
-      <c r="L70" s="911"/>
-      <c r="M70" s="911"/>
-      <c r="N70" s="911"/>
+      <c r="B70" s="897"/>
+      <c r="C70" s="897"/>
+      <c r="D70" s="897"/>
+      <c r="E70" s="897"/>
+      <c r="F70" s="897"/>
+      <c r="G70" s="897"/>
+      <c r="H70" s="897"/>
+      <c r="I70" s="897"/>
+      <c r="J70" s="897"/>
+      <c r="K70" s="897"/>
+      <c r="L70" s="897"/>
+      <c r="M70" s="897"/>
+      <c r="N70" s="897"/>
     </row>
     <row r="71" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="911" t="s">
+      <c r="A71" s="897" t="s">
         <v>340</v>
       </c>
-      <c r="B71" s="911"/>
-      <c r="C71" s="911"/>
-      <c r="D71" s="911"/>
-      <c r="E71" s="911"/>
-      <c r="F71" s="911"/>
-      <c r="G71" s="911"/>
-      <c r="H71" s="911"/>
-      <c r="I71" s="911"/>
-      <c r="J71" s="911"/>
-      <c r="K71" s="911"/>
-      <c r="L71" s="911"/>
-      <c r="M71" s="911"/>
-      <c r="N71" s="911"/>
+      <c r="B71" s="897"/>
+      <c r="C71" s="897"/>
+      <c r="D71" s="897"/>
+      <c r="E71" s="897"/>
+      <c r="F71" s="897"/>
+      <c r="G71" s="897"/>
+      <c r="H71" s="897"/>
+      <c r="I71" s="897"/>
+      <c r="J71" s="897"/>
+      <c r="K71" s="897"/>
+      <c r="L71" s="897"/>
+      <c r="M71" s="897"/>
+      <c r="N71" s="897"/>
     </row>
     <row r="72" spans="1:19" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="908" t="s">
+      <c r="A72" s="894" t="s">
         <v>341</v>
       </c>
-      <c r="B72" s="908"/>
-      <c r="C72" s="908"/>
-      <c r="D72" s="908"/>
-      <c r="E72" s="908"/>
-      <c r="F72" s="908"/>
-      <c r="G72" s="908"/>
-      <c r="H72" s="908"/>
-      <c r="I72" s="908"/>
-      <c r="J72" s="908"/>
-      <c r="K72" s="908"/>
-      <c r="L72" s="908"/>
-      <c r="M72" s="908"/>
-      <c r="N72" s="908"/>
+      <c r="B72" s="894"/>
+      <c r="C72" s="894"/>
+      <c r="D72" s="894"/>
+      <c r="E72" s="894"/>
+      <c r="F72" s="894"/>
+      <c r="G72" s="894"/>
+      <c r="H72" s="894"/>
+      <c r="I72" s="894"/>
+      <c r="J72" s="894"/>
+      <c r="K72" s="894"/>
+      <c r="L72" s="894"/>
+      <c r="M72" s="894"/>
+      <c r="N72" s="894"/>
     </row>
     <row r="73" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="294"/>
@@ -18784,10 +18784,10 @@
       <c r="A76" s="294"/>
       <c r="B76" s="294"/>
       <c r="C76" s="294"/>
-      <c r="K76" s="907"/>
-      <c r="L76" s="907"/>
-      <c r="M76" s="907"/>
-      <c r="N76" s="907"/>
+      <c r="K76" s="889"/>
+      <c r="L76" s="889"/>
+      <c r="M76" s="889"/>
+      <c r="N76" s="889"/>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="294"/>
@@ -18862,20 +18862,20 @@
       <c r="N84" s="295"/>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A85" s="915"/>
-      <c r="B85" s="915"/>
-      <c r="C85" s="915"/>
-      <c r="D85" s="915"/>
-      <c r="E85" s="915"/>
-      <c r="F85" s="915"/>
-      <c r="G85" s="915"/>
-      <c r="H85" s="915"/>
-      <c r="I85" s="915"/>
-      <c r="J85" s="915"/>
-      <c r="K85" s="915"/>
-      <c r="L85" s="915"/>
-      <c r="M85" s="915"/>
-      <c r="N85" s="915"/>
+      <c r="A85" s="891"/>
+      <c r="B85" s="891"/>
+      <c r="C85" s="891"/>
+      <c r="D85" s="891"/>
+      <c r="E85" s="891"/>
+      <c r="F85" s="891"/>
+      <c r="G85" s="891"/>
+      <c r="H85" s="891"/>
+      <c r="I85" s="891"/>
+      <c r="J85" s="891"/>
+      <c r="K85" s="891"/>
+      <c r="L85" s="891"/>
+      <c r="M85" s="891"/>
+      <c r="N85" s="891"/>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="92" t="s">
@@ -18890,10 +18890,10 @@
       <c r="H86" s="205"/>
       <c r="I86" s="205"/>
       <c r="J86" s="205"/>
-      <c r="K86" s="907"/>
-      <c r="L86" s="907"/>
-      <c r="M86" s="907"/>
-      <c r="N86" s="907"/>
+      <c r="K86" s="889"/>
+      <c r="L86" s="889"/>
+      <c r="M86" s="889"/>
+      <c r="N86" s="889"/>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="92" t="s">
@@ -18908,12 +18908,12 @@
       <c r="H87" s="205"/>
       <c r="I87" s="205"/>
       <c r="J87" s="205"/>
-      <c r="K87" s="907" t="s">
+      <c r="K87" s="889" t="s">
         <v>220</v>
       </c>
-      <c r="L87" s="907"/>
-      <c r="M87" s="907"/>
-      <c r="N87" s="907"/>
+      <c r="L87" s="889"/>
+      <c r="M87" s="889"/>
+      <c r="N87" s="889"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="205"/>
@@ -18986,12 +18986,42 @@
     <protectedRange sqref="E5:F6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="57">
-    <mergeCell ref="K87:N87"/>
-    <mergeCell ref="K54:N54"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="K86:N86"/>
-    <mergeCell ref="A85:N85"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="K52:N52"/>
+    <mergeCell ref="K53:N53"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="AB8:AD8"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="A11:N11"/>
+    <mergeCell ref="V20:X20"/>
+    <mergeCell ref="Y20:Z20"/>
+    <mergeCell ref="Y19:Z19"/>
+    <mergeCell ref="V19:X19"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="X42:Y42"/>
     <mergeCell ref="K76:N76"/>
     <mergeCell ref="I64:J64"/>
@@ -19007,42 +19037,12 @@
     <mergeCell ref="A68:N68"/>
     <mergeCell ref="A69:N69"/>
     <mergeCell ref="A71:N71"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="AB8:AD8"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="V20:X20"/>
-    <mergeCell ref="Y20:Z20"/>
-    <mergeCell ref="Y19:Z19"/>
-    <mergeCell ref="V19:X19"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="K52:N52"/>
-    <mergeCell ref="K53:N53"/>
+    <mergeCell ref="K87:N87"/>
+    <mergeCell ref="K54:N54"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="K86:N86"/>
+    <mergeCell ref="A85:N85"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.98425196850393704" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -19072,34 +19072,34 @@
   <sheetData>
     <row r="1" spans="1:12" ht="7.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="928" t="s">
+      <c r="B2" s="922" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="928"/>
-      <c r="D2" s="928"/>
-      <c r="E2" s="928"/>
-      <c r="F2" s="928"/>
-      <c r="G2" s="928"/>
-      <c r="H2" s="928"/>
-      <c r="I2" s="928"/>
-      <c r="J2" s="928"/>
-      <c r="K2" s="928"/>
-      <c r="L2" s="928"/>
+      <c r="C2" s="922"/>
+      <c r="D2" s="922"/>
+      <c r="E2" s="922"/>
+      <c r="F2" s="922"/>
+      <c r="G2" s="922"/>
+      <c r="H2" s="922"/>
+      <c r="I2" s="922"/>
+      <c r="J2" s="922"/>
+      <c r="K2" s="922"/>
+      <c r="L2" s="922"/>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="928" t="s">
+      <c r="B3" s="922" t="s">
         <v>236</v>
       </c>
-      <c r="C3" s="928"/>
-      <c r="D3" s="928"/>
-      <c r="E3" s="928"/>
-      <c r="F3" s="928"/>
-      <c r="G3" s="928"/>
-      <c r="H3" s="928"/>
-      <c r="I3" s="928"/>
-      <c r="J3" s="928"/>
-      <c r="K3" s="928"/>
-      <c r="L3" s="928"/>
+      <c r="C3" s="922"/>
+      <c r="D3" s="922"/>
+      <c r="E3" s="922"/>
+      <c r="F3" s="922"/>
+      <c r="G3" s="922"/>
+      <c r="H3" s="922"/>
+      <c r="I3" s="922"/>
+      <c r="J3" s="922"/>
+      <c r="K3" s="922"/>
+      <c r="L3" s="922"/>
     </row>
     <row r="4" spans="1:12" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="311"/>
@@ -19211,45 +19211,45 @@
     </row>
     <row r="11" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="255"/>
-      <c r="B11" s="927" t="s">
+      <c r="B11" s="921" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="796" t="s">
+      <c r="C11" s="808" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="796"/>
-      <c r="E11" s="796"/>
-      <c r="F11" s="796"/>
-      <c r="G11" s="796"/>
-      <c r="H11" s="796"/>
-      <c r="I11" s="796" t="s">
+      <c r="D11" s="808"/>
+      <c r="E11" s="808"/>
+      <c r="F11" s="808"/>
+      <c r="G11" s="808"/>
+      <c r="H11" s="808"/>
+      <c r="I11" s="808" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="796"/>
-      <c r="K11" s="796"/>
-      <c r="L11" s="796"/>
+      <c r="J11" s="808"/>
+      <c r="K11" s="808"/>
+      <c r="L11" s="808"/>
     </row>
     <row r="12" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="255"/>
-      <c r="B12" s="927"/>
-      <c r="C12" s="919" t="s">
+      <c r="B12" s="921"/>
+      <c r="C12" s="927" t="s">
         <v>198</v>
       </c>
-      <c r="D12" s="919"/>
-      <c r="E12" s="919"/>
-      <c r="F12" s="919"/>
-      <c r="G12" s="919"/>
-      <c r="H12" s="919"/>
-      <c r="I12" s="919" t="s">
+      <c r="D12" s="927"/>
+      <c r="E12" s="927"/>
+      <c r="F12" s="927"/>
+      <c r="G12" s="927"/>
+      <c r="H12" s="927"/>
+      <c r="I12" s="927" t="s">
         <v>198</v>
       </c>
-      <c r="J12" s="919"/>
-      <c r="K12" s="919"/>
-      <c r="L12" s="919"/>
+      <c r="J12" s="927"/>
+      <c r="K12" s="927"/>
+      <c r="L12" s="927"/>
     </row>
     <row r="13" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="255"/>
-      <c r="B13" s="927"/>
+      <c r="B13" s="921"/>
       <c r="C13" s="250" t="s">
         <v>196</v>
       </c>
@@ -19747,13 +19747,13 @@
       <c r="F24" s="83"/>
       <c r="G24" s="83"/>
       <c r="H24" s="83"/>
-      <c r="I24" s="929" t="e">
+      <c r="I24" s="923" t="e">
         <f>+AVERAGE(J23,L23)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="929"/>
-      <c r="K24" s="929"/>
-      <c r="L24" s="929"/>
+      <c r="J24" s="923"/>
+      <c r="K24" s="923"/>
+      <c r="L24" s="923"/>
       <c r="N24" s="264"/>
       <c r="O24" s="263"/>
       <c r="P24" s="263"/>
@@ -19873,13 +19873,13 @@
       </c>
       <c r="G29" s="209"/>
       <c r="H29" s="209"/>
-      <c r="I29" s="924" t="s">
+      <c r="I29" s="918" t="s">
         <v>217</v>
       </c>
-      <c r="J29" s="925"/>
-      <c r="K29" s="925"/>
-      <c r="L29" s="925"/>
-      <c r="M29" s="926"/>
+      <c r="J29" s="919"/>
+      <c r="K29" s="919"/>
+      <c r="L29" s="919"/>
+      <c r="M29" s="920"/>
       <c r="O29" s="209"/>
       <c r="P29" s="209"/>
       <c r="R29" s="209"/>
@@ -19901,15 +19901,15 @@
       </c>
       <c r="G30" s="209"/>
       <c r="H30" s="209"/>
-      <c r="I30" s="920" t="s">
+      <c r="I30" s="928" t="s">
         <v>212</v>
       </c>
-      <c r="J30" s="921"/>
-      <c r="K30" s="920" t="s">
+      <c r="J30" s="929"/>
+      <c r="K30" s="928" t="s">
         <v>213</v>
       </c>
-      <c r="L30" s="921"/>
-      <c r="M30" s="922" t="s">
+      <c r="L30" s="929"/>
+      <c r="M30" s="916" t="s">
         <v>214</v>
       </c>
       <c r="O30" s="209"/>
@@ -19945,7 +19945,7 @@
       <c r="L31" s="275" t="s">
         <v>216</v>
       </c>
-      <c r="M31" s="923"/>
+      <c r="M31" s="917"/>
       <c r="O31" s="209"/>
       <c r="P31" s="209"/>
       <c r="R31" s="209"/>
@@ -20112,12 +20112,12 @@
         <f>RSQ(D30:D32,B30:B32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D40" s="916" t="e">
+      <c r="D40" s="924" t="e">
         <f>IF(C40&lt;=0.95,"NO CONFORME","CONFORME")</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E40" s="917"/>
-      <c r="F40" s="918"/>
+      <c r="E40" s="925"/>
+      <c r="F40" s="926"/>
       <c r="G40" s="209"/>
       <c r="H40" s="257"/>
       <c r="I40" s="257"/>
@@ -20189,12 +20189,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="QbK/P4ukgbZU85pj93hV0ftn6ZZr2hJ3Xae2c00zbnGLirnsM7iT5h3St32dri55u5WTm1SV+UiG1Ty1N6MUfA==" saltValue="z/psz9/vsbYUqIhFhYyGLg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="M30:M31"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:L3"/>
-    <mergeCell ref="I24:L24"/>
     <mergeCell ref="D40:F40"/>
     <mergeCell ref="I11:L11"/>
     <mergeCell ref="C11:H11"/>
@@ -20202,6 +20196,12 @@
     <mergeCell ref="I12:L12"/>
     <mergeCell ref="I30:J30"/>
     <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M30:M31"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="I24:L24"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C12 I12" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -23277,18 +23277,18 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="959" t="s">
+      <c r="B19" s="953" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="959"/>
-      <c r="D19" s="959"/>
-      <c r="E19" s="959"/>
+      <c r="C19" s="953"/>
+      <c r="D19" s="953"/>
+      <c r="E19" s="953"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="328"/>
-      <c r="B20" s="953"/>
-      <c r="C20" s="953"/>
-      <c r="D20" s="953"/>
+      <c r="B20" s="958"/>
+      <c r="C20" s="958"/>
+      <c r="D20" s="958"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="236"/>
@@ -23339,20 +23339,20 @@
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="340"/>
-      <c r="B24" s="956" t="s">
+      <c r="B24" s="963" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="957"/>
-      <c r="D24" s="957"/>
-      <c r="E24" s="957"/>
-      <c r="F24" s="957"/>
-      <c r="G24" s="958"/>
-      <c r="H24" s="956" t="s">
+      <c r="C24" s="964"/>
+      <c r="D24" s="964"/>
+      <c r="E24" s="964"/>
+      <c r="F24" s="964"/>
+      <c r="G24" s="965"/>
+      <c r="H24" s="963" t="s">
         <v>144</v>
       </c>
-      <c r="I24" s="957"/>
-      <c r="J24" s="957"/>
-      <c r="K24" s="958"/>
+      <c r="I24" s="964"/>
+      <c r="J24" s="964"/>
+      <c r="K24" s="965"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="353" t="s">
@@ -23515,10 +23515,10 @@
       <c r="B29" s="330"/>
       <c r="C29" s="332"/>
       <c r="D29" s="330"/>
-      <c r="F29" s="953"/>
-      <c r="G29" s="953"/>
-      <c r="H29" s="953"/>
-      <c r="I29" s="953"/>
+      <c r="F29" s="958"/>
+      <c r="G29" s="958"/>
+      <c r="H29" s="958"/>
+      <c r="I29" s="958"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H30" s="350"/>
@@ -23526,17 +23526,17 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="328"/>
-      <c r="C31" s="963" t="s">
+      <c r="C31" s="959" t="s">
         <v>182</v>
       </c>
-      <c r="D31" s="964"/>
-      <c r="E31" s="965"/>
-      <c r="G31" s="955" t="s">
+      <c r="D31" s="960"/>
+      <c r="E31" s="961"/>
+      <c r="G31" s="957" t="s">
         <v>189</v>
       </c>
-      <c r="H31" s="955"/>
-      <c r="I31" s="955"/>
-      <c r="J31" s="955"/>
+      <c r="H31" s="957"/>
+      <c r="I31" s="957"/>
+      <c r="J31" s="957"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C32" s="335" t="s">
@@ -23562,7 +23562,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="954"/>
+      <c r="A33" s="962"/>
       <c r="C33" s="469">
         <v>1</v>
       </c>
@@ -23574,7 +23574,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="954"/>
+      <c r="A34" s="962"/>
       <c r="C34" s="469">
         <v>2</v>
       </c>
@@ -23586,7 +23586,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="954"/>
+      <c r="A35" s="962"/>
       <c r="C35" s="469">
         <v>3</v>
       </c>
@@ -23598,7 +23598,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="954"/>
+      <c r="A36" s="962"/>
       <c r="C36" s="469">
         <v>4</v>
       </c>
@@ -23610,7 +23610,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="960"/>
+      <c r="A37" s="954"/>
       <c r="C37" s="469">
         <v>5</v>
       </c>
@@ -23622,7 +23622,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="960"/>
+      <c r="A38" s="954"/>
       <c r="C38" s="469">
         <v>6</v>
       </c>
@@ -23634,7 +23634,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="960"/>
+      <c r="A39" s="954"/>
       <c r="C39" s="469">
         <v>7</v>
       </c>
@@ -23646,7 +23646,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="960"/>
+      <c r="A40" s="954"/>
       <c r="C40" s="469">
         <v>8</v>
       </c>
@@ -23801,39 +23801,40 @@
         <f>COUNT(C33:C52)</f>
         <v>20</v>
       </c>
-      <c r="C54" s="961" t="s">
+      <c r="C54" s="955" t="s">
         <v>186</v>
       </c>
-      <c r="D54" s="962"/>
+      <c r="D54" s="956"/>
       <c r="E54" s="582">
         <f>+STDEV(E33:E53)</f>
         <v>0.67082039324993703</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B55" s="955" t="s">
+      <c r="B55" s="957" t="s">
         <v>246</v>
       </c>
-      <c r="C55" s="955"/>
-      <c r="D55" s="955"/>
+      <c r="C55" s="957"/>
+      <c r="D55" s="957"/>
       <c r="E55" s="582">
         <f>E54/SQRT(B54)</f>
         <v>0.15000000000000002</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="H24:K24"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="A37:A40"/>
     <mergeCell ref="C54:D54"/>
     <mergeCell ref="B55:D55"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="C31:E31"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="H24:K24"/>
   </mergeCells>
   <conditionalFormatting sqref="E53">
     <cfRule type="cellIs" priority="1" stopIfTrue="1" operator="between">
@@ -25317,9 +25318,9 @@
       <c r="A2" s="329"/>
       <c r="G2" s="329"/>
       <c r="M2" s="328"/>
-      <c r="N2" s="953"/>
-      <c r="O2" s="953"/>
-      <c r="P2" s="953"/>
+      <c r="N2" s="958"/>
+      <c r="O2" s="958"/>
+      <c r="P2" s="958"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="329" t="s">
@@ -25328,7 +25329,7 @@
       <c r="G3" s="329" t="s">
         <v>327</v>
       </c>
-      <c r="M3" s="954"/>
+      <c r="M3" s="962"/>
       <c r="N3" s="656"/>
       <c r="O3" s="656"/>
       <c r="P3" s="656"/>
@@ -25346,7 +25347,7 @@
       <c r="H4" s="334">
         <v>46070</v>
       </c>
-      <c r="M4" s="954"/>
+      <c r="M4" s="962"/>
       <c r="N4" s="656"/>
       <c r="O4" s="657"/>
       <c r="P4" s="657"/>
@@ -25356,7 +25357,7 @@
       <c r="B5" s="658"/>
       <c r="G5" s="329"/>
       <c r="H5" s="658"/>
-      <c r="M5" s="954"/>
+      <c r="M5" s="962"/>
       <c r="N5" s="330"/>
       <c r="O5" s="330"/>
       <c r="P5" s="330"/>

</xml_diff>

<commit_message>
chore(templates): upload updated CBR and LLP templates and ensure sheet protection remains intact
</commit_message>
<xml_diff>
--- a/app/templates/informes/LLP/1-INF.-N-000-26-SU23-LL-LP-V07.xlsx
+++ b/app/templates/informes/LLP/1-INF.-N-000-26-SU23-LL-LP-V07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\LLP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79D023E-EDD6-49DD-A89E-7FE6478C4C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75B3838-DD6C-4132-B976-777DC6449927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="737" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5385,6 +5385,105 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="23" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -5415,150 +5514,177 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="191" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="11" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="10" fontId="50" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="2" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5588,178 +5714,99 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="8" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="2" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="2" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="187" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="60" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="191" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="11" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -5786,55 +5833,29 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="187" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="60" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="34" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="27" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="2" fontId="78" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="78" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="78" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="59" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5865,27 +5886,6 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="78" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="78" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="78" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="59" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="2" borderId="20" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5955,6 +5955,24 @@
     <xf numFmtId="0" fontId="56" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="66" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="11" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="66" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5968,12 +5986,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5981,18 +5993,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="11" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -12891,35 +12891,35 @@
     </row>
     <row r="6" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="802" t="s">
+      <c r="A7" s="790" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="802"/>
-      <c r="C7" s="802"/>
-      <c r="D7" s="802"/>
-      <c r="E7" s="802"/>
-      <c r="F7" s="802"/>
-      <c r="G7" s="802"/>
-      <c r="H7" s="802"/>
-      <c r="I7" s="802"/>
-      <c r="J7" s="802"/>
-      <c r="K7" s="802"/>
+      <c r="B7" s="790"/>
+      <c r="C7" s="790"/>
+      <c r="D7" s="790"/>
+      <c r="E7" s="790"/>
+      <c r="F7" s="790"/>
+      <c r="G7" s="790"/>
+      <c r="H7" s="790"/>
+      <c r="I7" s="790"/>
+      <c r="J7" s="790"/>
+      <c r="K7" s="790"/>
     </row>
     <row r="8" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="797">
+      <c r="A8" s="782">
         <f>+K13</f>
         <v>10</v>
       </c>
-      <c r="B8" s="797"/>
-      <c r="C8" s="797"/>
-      <c r="D8" s="797"/>
-      <c r="E8" s="797"/>
-      <c r="F8" s="797"/>
-      <c r="G8" s="797"/>
-      <c r="H8" s="797"/>
-      <c r="I8" s="797"/>
-      <c r="J8" s="797"/>
-      <c r="K8" s="797"/>
+      <c r="B8" s="782"/>
+      <c r="C8" s="782"/>
+      <c r="D8" s="782"/>
+      <c r="E8" s="782"/>
+      <c r="F8" s="782"/>
+      <c r="G8" s="782"/>
+      <c r="H8" s="782"/>
+      <c r="I8" s="782"/>
+      <c r="J8" s="782"/>
+      <c r="K8" s="782"/>
     </row>
     <row r="9" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O9" s="26"/>
@@ -13030,8 +13030,8 @@
       <c r="M13" s="32"/>
       <c r="P13" s="36"/>
       <c r="Q13" s="36"/>
-      <c r="R13" s="809"/>
-      <c r="S13" s="809"/>
+      <c r="R13" s="797"/>
+      <c r="S13" s="797"/>
     </row>
     <row r="14" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="148" t="s">
@@ -13055,19 +13055,19 @@
       <c r="S14" s="42"/>
     </row>
     <row r="15" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="810" t="s">
+      <c r="A15" s="798" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="811"/>
-      <c r="C15" s="811"/>
-      <c r="D15" s="811"/>
-      <c r="E15" s="811"/>
-      <c r="F15" s="811"/>
-      <c r="G15" s="811"/>
-      <c r="H15" s="811"/>
-      <c r="I15" s="811"/>
-      <c r="J15" s="811"/>
-      <c r="K15" s="812"/>
+      <c r="B15" s="799"/>
+      <c r="C15" s="799"/>
+      <c r="D15" s="799"/>
+      <c r="E15" s="799"/>
+      <c r="F15" s="799"/>
+      <c r="G15" s="799"/>
+      <c r="H15" s="799"/>
+      <c r="I15" s="799"/>
+      <c r="J15" s="799"/>
+      <c r="K15" s="800"/>
       <c r="L15" s="32"/>
       <c r="M15" s="32"/>
       <c r="P15" s="36"/>
@@ -13076,19 +13076,19 @@
       <c r="S15" s="42"/>
     </row>
     <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="814" t="s">
+      <c r="A16" s="802" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="815"/>
-      <c r="C16" s="815"/>
-      <c r="D16" s="815"/>
-      <c r="E16" s="815"/>
-      <c r="F16" s="815"/>
-      <c r="G16" s="815"/>
-      <c r="H16" s="815"/>
-      <c r="I16" s="815"/>
-      <c r="J16" s="815"/>
-      <c r="K16" s="816"/>
+      <c r="B16" s="803"/>
+      <c r="C16" s="803"/>
+      <c r="D16" s="803"/>
+      <c r="E16" s="803"/>
+      <c r="F16" s="803"/>
+      <c r="G16" s="803"/>
+      <c r="H16" s="803"/>
+      <c r="I16" s="803"/>
+      <c r="J16" s="803"/>
+      <c r="K16" s="804"/>
       <c r="L16" s="32"/>
       <c r="M16" s="32"/>
       <c r="N16" s="23" t="s">
@@ -13100,10 +13100,10 @@
       <c r="S16" s="42"/>
     </row>
     <row r="17" spans="1:30" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="798" t="s">
+      <c r="A17" s="783" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="799"/>
+      <c r="B17" s="784"/>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="44"/>
@@ -13148,8 +13148,8 @@
       <c r="AD17" s="118"/>
     </row>
     <row r="18" spans="1:30" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="800"/>
-      <c r="B18" s="801"/>
+      <c r="A18" s="785"/>
+      <c r="B18" s="786"/>
       <c r="C18" s="145"/>
       <c r="D18" s="145"/>
       <c r="E18" s="145"/>
@@ -13301,10 +13301,10 @@
       <c r="T20" s="128" t="s">
         <v>50</v>
       </c>
-      <c r="U20" s="796">
+      <c r="U20" s="781">
         <v>44090</v>
       </c>
-      <c r="V20" s="796"/>
+      <c r="V20" s="781"/>
       <c r="W20" s="129"/>
       <c r="X20" s="130"/>
       <c r="Y20" s="129"/>
@@ -13398,8 +13398,8 @@
     </row>
     <row r="23" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="52"/>
-      <c r="I23" s="803"/>
-      <c r="J23" s="803"/>
+      <c r="I23" s="791"/>
+      <c r="J23" s="791"/>
       <c r="K23" s="53"/>
       <c r="L23" s="32"/>
       <c r="M23" s="54"/>
@@ -13407,44 +13407,44 @@
     </row>
     <row r="24" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="56"/>
-      <c r="D24" s="805" t="s">
+      <c r="D24" s="793" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="806"/>
-      <c r="F24" s="806"/>
-      <c r="G24" s="807" t="s">
+      <c r="E24" s="794"/>
+      <c r="F24" s="794"/>
+      <c r="G24" s="795" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="808"/>
-      <c r="I24" s="804"/>
-      <c r="J24" s="804"/>
+      <c r="H24" s="796"/>
+      <c r="I24" s="792"/>
+      <c r="J24" s="792"/>
       <c r="K24" s="57"/>
       <c r="L24" s="32"/>
       <c r="M24" s="58"/>
       <c r="N24" s="138" t="s">
         <v>52</v>
       </c>
-      <c r="O24" s="817" t="s">
+      <c r="O24" s="805" t="s">
         <v>35</v>
       </c>
-      <c r="P24" s="819"/>
+      <c r="P24" s="807"/>
       <c r="Q24" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="R24" s="817" t="s">
+      <c r="R24" s="805" t="s">
         <v>34</v>
       </c>
-      <c r="S24" s="818"/>
+      <c r="S24" s="806"/>
       <c r="T24" s="59" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="793" t="s">
+      <c r="A25" s="808" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="794"/>
-      <c r="C25" s="795"/>
+      <c r="B25" s="809"/>
+      <c r="C25" s="810"/>
       <c r="D25" s="60">
         <f>IF($Q$24="NO","",O25)</f>
         <v>1</v>
@@ -13465,8 +13465,8 @@
         <f>IF($T$24="NO","",S25)</f>
         <v>2</v>
       </c>
-      <c r="I25" s="804"/>
-      <c r="J25" s="804"/>
+      <c r="I25" s="792"/>
+      <c r="J25" s="792"/>
       <c r="K25" s="57"/>
       <c r="L25" s="32"/>
       <c r="M25" s="58"/>
@@ -13490,11 +13490,11 @@
       </c>
     </row>
     <row r="26" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="790" t="s">
+      <c r="A26" s="787" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="791"/>
-      <c r="C26" s="792"/>
+      <c r="B26" s="788"/>
+      <c r="C26" s="789"/>
       <c r="D26" s="66">
         <f>IF($Q$24="NO","",O26)</f>
         <v>5</v>
@@ -13515,8 +13515,8 @@
         <f>IF($T$24="NO","",S26)</f>
         <v>10</v>
       </c>
-      <c r="I26" s="813"/>
-      <c r="J26" s="813"/>
+      <c r="I26" s="801"/>
+      <c r="J26" s="801"/>
       <c r="K26" s="69"/>
       <c r="L26" s="70"/>
       <c r="M26" s="58"/>
@@ -13545,11 +13545,11 @@
       </c>
     </row>
     <row r="27" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="790" t="s">
+      <c r="A27" s="787" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="791"/>
-      <c r="C27" s="792"/>
+      <c r="B27" s="788"/>
+      <c r="C27" s="789"/>
       <c r="D27" s="66">
         <f t="shared" ref="D27:D29" si="2">IF($Q$24="NO","",O27)</f>
         <v>34</v>
@@ -13588,11 +13588,11 @@
       <c r="S27" s="136"/>
     </row>
     <row r="28" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="790" t="s">
+      <c r="A28" s="787" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="791"/>
-      <c r="C28" s="792"/>
+      <c r="B28" s="788"/>
+      <c r="C28" s="789"/>
       <c r="D28" s="86">
         <f t="shared" si="2"/>
         <v>45.749976347249998</v>
@@ -13643,11 +13643,11 @@
       </c>
     </row>
     <row r="29" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="790" t="s">
+      <c r="A29" s="787" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="791"/>
-      <c r="C29" s="792"/>
+      <c r="B29" s="788"/>
+      <c r="C29" s="789"/>
       <c r="D29" s="86">
         <f t="shared" si="2"/>
         <v>41.369978611709996</v>
@@ -13698,11 +13698,11 @@
       </c>
     </row>
     <row r="30" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="790" t="s">
+      <c r="A30" s="787" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="791"/>
-      <c r="C30" s="792"/>
+      <c r="B30" s="788"/>
+      <c r="C30" s="789"/>
       <c r="D30" s="86">
         <f t="shared" ref="D30:F33" si="10">IF($Q$24="NO","",O31)</f>
         <v>22.739988243419997</v>
@@ -13753,11 +13753,11 @@
       </c>
     </row>
     <row r="31" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="790" t="s">
+      <c r="A31" s="787" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="791"/>
-      <c r="C31" s="792"/>
+      <c r="B31" s="788"/>
+      <c r="C31" s="789"/>
       <c r="D31" s="86">
         <f t="shared" si="10"/>
         <v>4.3799977355400017</v>
@@ -13808,11 +13808,11 @@
       </c>
     </row>
     <row r="32" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="790" t="s">
+      <c r="A32" s="787" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="791"/>
-      <c r="C32" s="792"/>
+      <c r="B32" s="788"/>
+      <c r="C32" s="789"/>
       <c r="D32" s="86">
         <f t="shared" si="10"/>
         <v>18.629990368289999</v>
@@ -13863,11 +13863,11 @@
       </c>
     </row>
     <row r="33" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="793" t="s">
+      <c r="A33" s="808" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="794"/>
-      <c r="C33" s="795"/>
+      <c r="B33" s="809"/>
+      <c r="C33" s="810"/>
       <c r="D33" s="86">
         <f t="shared" si="10"/>
         <v>23.510466988727867</v>
@@ -13977,10 +13977,10 @@
       <c r="D36" s="17"/>
       <c r="E36" s="17"/>
       <c r="F36" s="17"/>
-      <c r="G36" s="781" t="s">
+      <c r="G36" s="811" t="s">
         <v>75</v>
       </c>
-      <c r="H36" s="782"/>
+      <c r="H36" s="812"/>
       <c r="I36" s="152">
         <f>+IF(Q24="NO","NP",ROUND(O49,0))</f>
         <v>24</v>
@@ -14034,10 +14034,10 @@
       <c r="D38" s="17"/>
       <c r="E38" s="17"/>
       <c r="F38" s="17"/>
-      <c r="G38" s="781" t="s">
+      <c r="G38" s="811" t="s">
         <v>76</v>
       </c>
-      <c r="H38" s="782"/>
+      <c r="H38" s="812"/>
       <c r="I38" s="152">
         <f>+IF(T24="NO","NP",ROUND(O42,0))</f>
         <v>13</v>
@@ -14089,10 +14089,10 @@
       <c r="D40" s="19"/>
       <c r="E40" s="19"/>
       <c r="F40" s="19"/>
-      <c r="G40" s="781" t="s">
+      <c r="G40" s="811" t="s">
         <v>77</v>
       </c>
-      <c r="H40" s="782"/>
+      <c r="H40" s="812"/>
       <c r="I40" s="152">
         <f>IF(T24="NO","NP",I36-I38)</f>
         <v>11</v>
@@ -14474,12 +14474,12 @@
       <c r="E57" s="168"/>
       <c r="F57" s="169"/>
       <c r="G57" s="169"/>
-      <c r="H57" s="786" t="s">
+      <c r="H57" s="816" t="s">
         <v>101</v>
       </c>
-      <c r="I57" s="787"/>
-      <c r="J57" s="787"/>
-      <c r="K57" s="788"/>
+      <c r="I57" s="817"/>
+      <c r="J57" s="817"/>
+      <c r="K57" s="818"/>
       <c r="L57" s="32"/>
       <c r="M57" s="32"/>
     </row>
@@ -14493,31 +14493,31 @@
       <c r="E58" s="168"/>
       <c r="F58" s="169"/>
       <c r="G58" s="169"/>
-      <c r="H58" s="786" t="s">
+      <c r="H58" s="816" t="s">
         <v>102</v>
       </c>
-      <c r="I58" s="787"/>
-      <c r="J58" s="787"/>
-      <c r="K58" s="788"/>
+      <c r="I58" s="817"/>
+      <c r="J58" s="817"/>
+      <c r="K58" s="818"/>
       <c r="L58" s="32"/>
       <c r="M58" s="32"/>
     </row>
     <row r="59" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="785" t="s">
+      <c r="A59" s="815" t="s">
         <v>84</v>
       </c>
-      <c r="B59" s="785"/>
-      <c r="C59" s="785"/>
-      <c r="D59" s="785"/>
-      <c r="E59" s="785"/>
-      <c r="F59" s="785"/>
-      <c r="G59" s="785"/>
-      <c r="H59" s="786">
+      <c r="B59" s="815"/>
+      <c r="C59" s="815"/>
+      <c r="D59" s="815"/>
+      <c r="E59" s="815"/>
+      <c r="F59" s="815"/>
+      <c r="G59" s="815"/>
+      <c r="H59" s="816">
         <v>23</v>
       </c>
-      <c r="I59" s="787"/>
-      <c r="J59" s="787"/>
-      <c r="K59" s="788"/>
+      <c r="I59" s="817"/>
+      <c r="J59" s="817"/>
+      <c r="K59" s="818"/>
       <c r="L59" s="32"/>
       <c r="M59" s="32"/>
       <c r="N59" s="153"/>
@@ -14532,31 +14532,31 @@
       <c r="E60" s="168"/>
       <c r="F60" s="169"/>
       <c r="G60" s="169"/>
-      <c r="H60" s="786" t="s">
+      <c r="H60" s="816" t="s">
         <v>103</v>
       </c>
-      <c r="I60" s="787"/>
-      <c r="J60" s="787"/>
-      <c r="K60" s="788"/>
+      <c r="I60" s="817"/>
+      <c r="J60" s="817"/>
+      <c r="K60" s="818"/>
       <c r="L60" s="32"/>
       <c r="M60" s="32"/>
     </row>
     <row r="61" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="785" t="s">
+      <c r="A61" s="815" t="s">
         <v>86</v>
       </c>
-      <c r="B61" s="785"/>
-      <c r="C61" s="785"/>
-      <c r="D61" s="785"/>
-      <c r="E61" s="785"/>
-      <c r="F61" s="785"/>
-      <c r="G61" s="785"/>
-      <c r="H61" s="786" t="s">
+      <c r="B61" s="815"/>
+      <c r="C61" s="815"/>
+      <c r="D61" s="815"/>
+      <c r="E61" s="815"/>
+      <c r="F61" s="815"/>
+      <c r="G61" s="815"/>
+      <c r="H61" s="816" t="s">
         <v>104</v>
       </c>
-      <c r="I61" s="787"/>
-      <c r="J61" s="787"/>
-      <c r="K61" s="788"/>
+      <c r="I61" s="817"/>
+      <c r="J61" s="817"/>
+      <c r="K61" s="818"/>
       <c r="L61" s="32"/>
       <c r="M61" s="32"/>
     </row>
@@ -14586,13 +14586,13 @@
       <c r="B64" s="156"/>
       <c r="C64" s="156"/>
       <c r="D64" s="156"/>
-      <c r="H64" s="789"/>
-      <c r="I64" s="789"/>
-      <c r="J64" s="789"/>
-      <c r="K64" s="789"/>
-      <c r="L64" s="789"/>
-      <c r="M64" s="789"/>
-      <c r="N64" s="789"/>
+      <c r="H64" s="819"/>
+      <c r="I64" s="819"/>
+      <c r="J64" s="819"/>
+      <c r="K64" s="819"/>
+      <c r="L64" s="819"/>
+      <c r="M64" s="819"/>
+      <c r="N64" s="819"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="157" t="s">
@@ -14654,12 +14654,12 @@
       </c>
       <c r="B71" s="160"/>
       <c r="D71" s="161"/>
-      <c r="H71" s="784" t="s">
+      <c r="H71" s="814" t="s">
         <v>81</v>
       </c>
-      <c r="I71" s="784"/>
-      <c r="J71" s="784"/>
-      <c r="K71" s="784"/>
+      <c r="I71" s="814"/>
+      <c r="J71" s="814"/>
+      <c r="K71" s="814"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="18"/>
@@ -14679,32 +14679,32 @@
       </c>
     </row>
     <row r="75" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="783" t="s">
+      <c r="A75" s="813" t="s">
         <v>79</v>
       </c>
-      <c r="B75" s="783"/>
-      <c r="C75" s="783"/>
-      <c r="D75" s="783"/>
-      <c r="E75" s="783"/>
-      <c r="F75" s="783"/>
-      <c r="G75" s="783"/>
-      <c r="H75" s="783"/>
-      <c r="I75" s="783"/>
-      <c r="J75" s="783"/>
-      <c r="K75" s="783"/>
+      <c r="B75" s="813"/>
+      <c r="C75" s="813"/>
+      <c r="D75" s="813"/>
+      <c r="E75" s="813"/>
+      <c r="F75" s="813"/>
+      <c r="G75" s="813"/>
+      <c r="H75" s="813"/>
+      <c r="I75" s="813"/>
+      <c r="J75" s="813"/>
+      <c r="K75" s="813"/>
     </row>
     <row r="76" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="783"/>
-      <c r="B76" s="783"/>
-      <c r="C76" s="783"/>
-      <c r="D76" s="783"/>
-      <c r="E76" s="783"/>
-      <c r="F76" s="783"/>
-      <c r="G76" s="783"/>
-      <c r="H76" s="783"/>
-      <c r="I76" s="783"/>
-      <c r="J76" s="783"/>
-      <c r="K76" s="783"/>
+      <c r="A76" s="813"/>
+      <c r="B76" s="813"/>
+      <c r="C76" s="813"/>
+      <c r="D76" s="813"/>
+      <c r="E76" s="813"/>
+      <c r="F76" s="813"/>
+      <c r="G76" s="813"/>
+      <c r="H76" s="813"/>
+      <c r="I76" s="813"/>
+      <c r="J76" s="813"/>
+      <c r="K76" s="813"/>
     </row>
     <row r="78" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -14713,6 +14713,28 @@
     <protectedRange sqref="C10:C11" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="38">
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="H71:K71"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="H57:K57"/>
+    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="H64:N64"/>
+    <mergeCell ref="H58:K58"/>
+    <mergeCell ref="H60:K60"/>
+    <mergeCell ref="H61:K61"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="U20:V20"/>
     <mergeCell ref="A8:K8"/>
     <mergeCell ref="A17:B18"/>
@@ -14729,28 +14751,6 @@
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="R24:S24"/>
     <mergeCell ref="O24:P24"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="A76:K76"/>
-    <mergeCell ref="H71:K71"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A61:G61"/>
-    <mergeCell ref="H57:K57"/>
-    <mergeCell ref="H59:K59"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="H64:N64"/>
-    <mergeCell ref="H58:K58"/>
-    <mergeCell ref="H60:K60"/>
-    <mergeCell ref="H61:K61"/>
   </mergeCells>
   <conditionalFormatting sqref="A59">
     <cfRule type="cellIs" priority="2" stopIfTrue="1" operator="between">
@@ -14909,42 +14909,42 @@
       <c r="Q6" s="770"/>
     </row>
     <row r="7" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="881" t="s">
+      <c r="A7" s="823" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="881"/>
-      <c r="C7" s="881"/>
-      <c r="D7" s="881"/>
-      <c r="E7" s="881"/>
-      <c r="F7" s="881"/>
-      <c r="G7" s="881"/>
-      <c r="H7" s="881"/>
-      <c r="I7" s="881"/>
-      <c r="J7" s="881"/>
-      <c r="K7" s="881"/>
-      <c r="L7" s="881"/>
-      <c r="M7" s="881"/>
+      <c r="B7" s="823"/>
+      <c r="C7" s="823"/>
+      <c r="D7" s="823"/>
+      <c r="E7" s="823"/>
+      <c r="F7" s="823"/>
+      <c r="G7" s="823"/>
+      <c r="H7" s="823"/>
+      <c r="I7" s="823"/>
+      <c r="J7" s="823"/>
+      <c r="K7" s="823"/>
+      <c r="L7" s="823"/>
+      <c r="M7" s="823"/>
       <c r="P7" s="682" t="s">
         <v>269</v>
       </c>
       <c r="Q7" s="770"/>
     </row>
     <row r="8" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="882" t="s">
+      <c r="A8" s="824" t="s">
         <v>272</v>
       </c>
-      <c r="B8" s="882"/>
-      <c r="C8" s="882"/>
-      <c r="D8" s="882"/>
-      <c r="E8" s="882"/>
-      <c r="F8" s="882"/>
-      <c r="G8" s="882"/>
-      <c r="H8" s="882"/>
-      <c r="I8" s="882"/>
-      <c r="J8" s="882"/>
-      <c r="K8" s="882"/>
-      <c r="L8" s="882"/>
-      <c r="M8" s="882"/>
+      <c r="B8" s="824"/>
+      <c r="C8" s="824"/>
+      <c r="D8" s="824"/>
+      <c r="E8" s="824"/>
+      <c r="F8" s="824"/>
+      <c r="G8" s="824"/>
+      <c r="H8" s="824"/>
+      <c r="I8" s="824"/>
+      <c r="J8" s="824"/>
+      <c r="K8" s="824"/>
+      <c r="L8" s="824"/>
+      <c r="M8" s="824"/>
       <c r="P8" s="682" t="s">
         <v>319</v>
       </c>
@@ -14971,23 +14971,23 @@
     </row>
     <row r="10" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="679"/>
-      <c r="C10" s="883" t="s">
+      <c r="C10" s="825" t="s">
         <v>273</v>
       </c>
-      <c r="D10" s="883"/>
-      <c r="E10" s="883" t="s">
+      <c r="D10" s="825"/>
+      <c r="E10" s="825" t="s">
         <v>274</v>
       </c>
-      <c r="F10" s="883"/>
-      <c r="G10" s="883"/>
-      <c r="H10" s="883" t="s">
+      <c r="F10" s="825"/>
+      <c r="G10" s="825"/>
+      <c r="H10" s="825" t="s">
         <v>275</v>
       </c>
-      <c r="I10" s="883"/>
-      <c r="J10" s="883" t="s">
+      <c r="I10" s="825"/>
+      <c r="J10" s="825" t="s">
         <v>276</v>
       </c>
-      <c r="K10" s="883"/>
+      <c r="K10" s="825"/>
       <c r="L10" s="679"/>
       <c r="M10" s="679"/>
       <c r="N10" s="121"/>
@@ -14998,15 +14998,15 @@
     <row r="11" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="679"/>
       <c r="B11" s="679"/>
-      <c r="C11" s="884"/>
-      <c r="D11" s="884"/>
-      <c r="E11" s="884"/>
-      <c r="F11" s="884"/>
-      <c r="G11" s="884"/>
-      <c r="H11" s="885"/>
-      <c r="I11" s="884"/>
-      <c r="J11" s="884"/>
-      <c r="K11" s="884"/>
+      <c r="C11" s="826"/>
+      <c r="D11" s="826"/>
+      <c r="E11" s="826"/>
+      <c r="F11" s="826"/>
+      <c r="G11" s="826"/>
+      <c r="H11" s="827"/>
+      <c r="I11" s="826"/>
+      <c r="J11" s="826"/>
+      <c r="K11" s="826"/>
       <c r="L11" s="679"/>
       <c r="M11" s="679"/>
       <c r="N11" s="121"/>
@@ -15038,21 +15038,21 @@
       <c r="Q12" s="771"/>
     </row>
     <row r="13" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="886" t="s">
+      <c r="A13" s="828" t="s">
         <v>277</v>
       </c>
-      <c r="B13" s="887"/>
-      <c r="C13" s="887"/>
-      <c r="D13" s="887"/>
-      <c r="E13" s="887"/>
-      <c r="F13" s="887"/>
-      <c r="G13" s="887"/>
-      <c r="H13" s="887"/>
-      <c r="I13" s="887"/>
-      <c r="J13" s="887"/>
-      <c r="K13" s="887"/>
-      <c r="L13" s="887"/>
-      <c r="M13" s="888"/>
+      <c r="B13" s="829"/>
+      <c r="C13" s="829"/>
+      <c r="D13" s="829"/>
+      <c r="E13" s="829"/>
+      <c r="F13" s="829"/>
+      <c r="G13" s="829"/>
+      <c r="H13" s="829"/>
+      <c r="I13" s="829"/>
+      <c r="J13" s="829"/>
+      <c r="K13" s="829"/>
+      <c r="L13" s="829"/>
+      <c r="M13" s="830"/>
       <c r="N13" s="121"/>
       <c r="O13" s="121"/>
       <c r="P13" s="682" t="s">
@@ -15061,21 +15061,21 @@
       <c r="Q13" s="771"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="878" t="s">
+      <c r="A14" s="820" t="s">
         <v>236</v>
       </c>
-      <c r="B14" s="879"/>
-      <c r="C14" s="879"/>
-      <c r="D14" s="879"/>
-      <c r="E14" s="879"/>
-      <c r="F14" s="879"/>
-      <c r="G14" s="879"/>
-      <c r="H14" s="879"/>
-      <c r="I14" s="879"/>
-      <c r="J14" s="879"/>
-      <c r="K14" s="879"/>
-      <c r="L14" s="879"/>
-      <c r="M14" s="880"/>
+      <c r="B14" s="821"/>
+      <c r="C14" s="821"/>
+      <c r="D14" s="821"/>
+      <c r="E14" s="821"/>
+      <c r="F14" s="821"/>
+      <c r="G14" s="821"/>
+      <c r="H14" s="821"/>
+      <c r="I14" s="821"/>
+      <c r="J14" s="821"/>
+      <c r="K14" s="821"/>
+      <c r="L14" s="821"/>
+      <c r="M14" s="822"/>
       <c r="N14" s="121"/>
       <c r="O14" s="121"/>
       <c r="P14" s="769"/>
@@ -15103,19 +15103,19 @@
       <c r="Q15" s="772"/>
     </row>
     <row r="16" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="860" t="s">
+      <c r="B16" s="832" t="s">
         <v>218</v>
       </c>
-      <c r="C16" s="861"/>
-      <c r="D16" s="861"/>
-      <c r="E16" s="861"/>
-      <c r="F16" s="861"/>
-      <c r="G16" s="861"/>
-      <c r="H16" s="861"/>
-      <c r="I16" s="861"/>
-      <c r="J16" s="861"/>
-      <c r="K16" s="861"/>
-      <c r="L16" s="862"/>
+      <c r="C16" s="833"/>
+      <c r="D16" s="833"/>
+      <c r="E16" s="833"/>
+      <c r="F16" s="833"/>
+      <c r="G16" s="833"/>
+      <c r="H16" s="833"/>
+      <c r="I16" s="833"/>
+      <c r="J16" s="833"/>
+      <c r="K16" s="833"/>
+      <c r="L16" s="834"/>
       <c r="M16" s="687"/>
       <c r="O16" s="121"/>
       <c r="P16" s="682" t="s">
@@ -15134,9 +15134,9 @@
       <c r="G17" s="689"/>
       <c r="H17" s="689"/>
       <c r="I17" s="690"/>
-      <c r="J17" s="863"/>
-      <c r="K17" s="863"/>
-      <c r="L17" s="863"/>
+      <c r="J17" s="835"/>
+      <c r="K17" s="835"/>
+      <c r="L17" s="835"/>
       <c r="M17" s="691"/>
       <c r="N17" s="692"/>
       <c r="O17" s="121"/>
@@ -15159,9 +15159,9 @@
       <c r="G18" s="694"/>
       <c r="H18" s="694"/>
       <c r="I18" s="695"/>
-      <c r="J18" s="863"/>
-      <c r="K18" s="863"/>
-      <c r="L18" s="863"/>
+      <c r="J18" s="835"/>
+      <c r="K18" s="835"/>
+      <c r="L18" s="835"/>
       <c r="M18" s="691"/>
       <c r="N18" s="692"/>
       <c r="O18" s="121"/>
@@ -15181,9 +15181,9 @@
       <c r="G19" s="689"/>
       <c r="H19" s="689"/>
       <c r="I19" s="690"/>
-      <c r="J19" s="863"/>
-      <c r="K19" s="863"/>
-      <c r="L19" s="863"/>
+      <c r="J19" s="835"/>
+      <c r="K19" s="835"/>
+      <c r="L19" s="835"/>
       <c r="M19" s="691"/>
       <c r="N19" s="692"/>
       <c r="O19" s="121"/>
@@ -15203,9 +15203,9 @@
       <c r="G20" s="697"/>
       <c r="H20" s="697"/>
       <c r="I20" s="698"/>
-      <c r="J20" s="863"/>
-      <c r="K20" s="863"/>
-      <c r="L20" s="863"/>
+      <c r="J20" s="835"/>
+      <c r="K20" s="835"/>
+      <c r="L20" s="835"/>
       <c r="M20" s="691"/>
       <c r="N20" s="692"/>
       <c r="O20" s="121"/>
@@ -15225,9 +15225,9 @@
       <c r="G21" s="689"/>
       <c r="H21" s="689"/>
       <c r="I21" s="690"/>
-      <c r="J21" s="864"/>
-      <c r="K21" s="865"/>
-      <c r="L21" s="866"/>
+      <c r="J21" s="836"/>
+      <c r="K21" s="837"/>
+      <c r="L21" s="838"/>
       <c r="M21" s="691"/>
       <c r="O21" s="121"/>
       <c r="P21" s="318"/>
@@ -15247,9 +15247,9 @@
       <c r="G22" s="697"/>
       <c r="H22" s="697"/>
       <c r="I22" s="698"/>
-      <c r="J22" s="867"/>
-      <c r="K22" s="868"/>
-      <c r="L22" s="869"/>
+      <c r="J22" s="839"/>
+      <c r="K22" s="840"/>
+      <c r="L22" s="841"/>
       <c r="M22" s="691"/>
       <c r="O22" s="121"/>
       <c r="P22" s="318"/>
@@ -15269,9 +15269,9 @@
       <c r="G23" s="689"/>
       <c r="H23" s="689"/>
       <c r="I23" s="690"/>
-      <c r="J23" s="870"/>
-      <c r="K23" s="871"/>
-      <c r="L23" s="872"/>
+      <c r="J23" s="842"/>
+      <c r="K23" s="843"/>
+      <c r="L23" s="844"/>
       <c r="M23" s="691"/>
       <c r="N23" s="692"/>
       <c r="O23" s="121"/>
@@ -15282,19 +15282,19 @@
       <c r="T23" s="317"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="873" t="s">
+      <c r="B24" s="845" t="s">
         <v>285</v>
       </c>
-      <c r="C24" s="874"/>
-      <c r="D24" s="874"/>
-      <c r="E24" s="874"/>
-      <c r="F24" s="874"/>
-      <c r="G24" s="874"/>
-      <c r="H24" s="874"/>
-      <c r="I24" s="874"/>
-      <c r="J24" s="874"/>
-      <c r="K24" s="874"/>
-      <c r="L24" s="875"/>
+      <c r="C24" s="846"/>
+      <c r="D24" s="846"/>
+      <c r="E24" s="846"/>
+      <c r="F24" s="846"/>
+      <c r="G24" s="846"/>
+      <c r="H24" s="846"/>
+      <c r="I24" s="846"/>
+      <c r="J24" s="846"/>
+      <c r="K24" s="846"/>
+      <c r="L24" s="847"/>
       <c r="M24" s="699"/>
       <c r="N24" s="692"/>
       <c r="O24" s="121"/>
@@ -15341,12 +15341,12 @@
       <c r="F26" s="705"/>
       <c r="G26" s="705"/>
       <c r="H26" s="702"/>
-      <c r="I26" s="876" t="s">
+      <c r="I26" s="848" t="s">
         <v>290</v>
       </c>
-      <c r="J26" s="876"/>
-      <c r="K26" s="876"/>
-      <c r="L26" s="877"/>
+      <c r="J26" s="848"/>
+      <c r="K26" s="848"/>
+      <c r="L26" s="849"/>
       <c r="M26" s="699"/>
       <c r="N26" s="692"/>
       <c r="O26" s="121"/>
@@ -15379,26 +15379,26 @@
       <c r="T27" s="317"/>
     </row>
     <row r="28" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="860" t="s">
+      <c r="B28" s="832" t="s">
         <v>291</v>
       </c>
-      <c r="C28" s="861"/>
-      <c r="D28" s="861"/>
-      <c r="E28" s="861"/>
-      <c r="F28" s="861"/>
-      <c r="G28" s="861"/>
-      <c r="H28" s="861"/>
-      <c r="I28" s="861"/>
-      <c r="J28" s="861"/>
-      <c r="K28" s="861"/>
-      <c r="L28" s="862"/>
+      <c r="C28" s="833"/>
+      <c r="D28" s="833"/>
+      <c r="E28" s="833"/>
+      <c r="F28" s="833"/>
+      <c r="G28" s="833"/>
+      <c r="H28" s="833"/>
+      <c r="I28" s="833"/>
+      <c r="J28" s="833"/>
+      <c r="K28" s="833"/>
+      <c r="L28" s="834"/>
       <c r="M28" s="709"/>
       <c r="N28" s="692"/>
-      <c r="O28" s="832" t="s">
+      <c r="O28" s="831" t="s">
         <v>35</v>
       </c>
-      <c r="P28" s="832"/>
-      <c r="Q28" s="832"/>
+      <c r="P28" s="831"/>
+      <c r="Q28" s="831"/>
       <c r="R28" s="317"/>
       <c r="S28" s="317"/>
       <c r="T28" s="317"/>
@@ -15414,9 +15414,9 @@
       <c r="G29" s="713"/>
       <c r="H29" s="713"/>
       <c r="I29" s="714"/>
-      <c r="J29" s="830"/>
+      <c r="J29" s="850"/>
       <c r="K29" s="854"/>
-      <c r="L29" s="831"/>
+      <c r="L29" s="851"/>
       <c r="M29" s="709"/>
       <c r="N29" s="692"/>
       <c r="O29" s="716" t="s">
@@ -15476,7 +15476,7 @@
       <c r="I31" s="714"/>
       <c r="J31" s="858"/>
       <c r="K31" s="854"/>
-      <c r="L31" s="831"/>
+      <c r="L31" s="851"/>
       <c r="M31" s="722"/>
       <c r="N31" s="692"/>
       <c r="O31" s="721" t="e">
@@ -15506,9 +15506,9 @@
       <c r="G32" s="713"/>
       <c r="H32" s="713"/>
       <c r="I32" s="714"/>
-      <c r="J32" s="830"/>
+      <c r="J32" s="850"/>
       <c r="K32" s="854"/>
-      <c r="L32" s="831"/>
+      <c r="L32" s="851"/>
       <c r="N32" s="692"/>
       <c r="O32" s="721" t="e">
         <f>+LN(P32)</f>
@@ -15534,9 +15534,9 @@
       <c r="G33" s="727"/>
       <c r="H33" s="727"/>
       <c r="I33" s="728"/>
-      <c r="J33" s="830"/>
+      <c r="J33" s="850"/>
       <c r="K33" s="854"/>
-      <c r="L33" s="831"/>
+      <c r="L33" s="851"/>
       <c r="N33" s="692"/>
       <c r="O33" s="729"/>
       <c r="P33" s="444" t="s">
@@ -15555,36 +15555,36 @@
       <c r="O34" s="731"/>
     </row>
     <row r="35" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="840" t="s">
+      <c r="B35" s="860" t="s">
         <v>297</v>
       </c>
-      <c r="C35" s="841"/>
-      <c r="D35" s="841"/>
-      <c r="E35" s="841"/>
-      <c r="F35" s="842"/>
-      <c r="G35" s="846" t="s">
+      <c r="C35" s="861"/>
+      <c r="D35" s="861"/>
+      <c r="E35" s="861"/>
+      <c r="F35" s="862"/>
+      <c r="G35" s="866" t="s">
         <v>35</v>
       </c>
-      <c r="H35" s="846"/>
-      <c r="I35" s="846"/>
-      <c r="J35" s="847"/>
-      <c r="K35" s="848" t="s">
+      <c r="H35" s="866"/>
+      <c r="I35" s="866"/>
+      <c r="J35" s="867"/>
+      <c r="K35" s="868" t="s">
         <v>34</v>
       </c>
-      <c r="L35" s="846"/>
+      <c r="L35" s="866"/>
       <c r="M35" s="732"/>
       <c r="N35" s="692"/>
     </row>
     <row r="36" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="843"/>
-      <c r="C36" s="844"/>
-      <c r="D36" s="844"/>
-      <c r="E36" s="844"/>
-      <c r="F36" s="845"/>
-      <c r="G36" s="849">
+      <c r="B36" s="863"/>
+      <c r="C36" s="864"/>
+      <c r="D36" s="864"/>
+      <c r="E36" s="864"/>
+      <c r="F36" s="865"/>
+      <c r="G36" s="869">
         <v>1</v>
       </c>
-      <c r="H36" s="850"/>
+      <c r="H36" s="870"/>
       <c r="I36" s="734">
         <v>2</v>
       </c>
@@ -15599,11 +15599,11 @@
       </c>
       <c r="M36" s="732"/>
       <c r="N36" s="692"/>
-      <c r="O36" s="851" t="s">
+      <c r="O36" s="871" t="s">
         <v>244</v>
       </c>
-      <c r="P36" s="852"/>
-      <c r="Q36" s="853"/>
+      <c r="P36" s="872"/>
+      <c r="Q36" s="873"/>
       <c r="R36" s="729"/>
       <c r="S36" s="729"/>
     </row>
@@ -15617,8 +15617,8 @@
       <c r="D37" s="739"/>
       <c r="E37" s="739"/>
       <c r="F37" s="740"/>
-      <c r="G37" s="830"/>
-      <c r="H37" s="831"/>
+      <c r="G37" s="850"/>
+      <c r="H37" s="851"/>
       <c r="I37" s="737"/>
       <c r="J37" s="715"/>
       <c r="K37" s="741"/>
@@ -15629,11 +15629,11 @@
         <f>RSQ(Q30:Q32,O30:O32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="P37" s="828" t="e">
+      <c r="P37" s="852" t="e">
         <f>IF(O37&lt;=0.95,"NO CONFORME","CONFORME")</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Q37" s="829"/>
+      <c r="Q37" s="853"/>
       <c r="R37" s="729"/>
       <c r="S37" s="729"/>
     </row>
@@ -15647,8 +15647,8 @@
       <c r="D38" s="739"/>
       <c r="E38" s="739"/>
       <c r="F38" s="740"/>
-      <c r="G38" s="830"/>
-      <c r="H38" s="831"/>
+      <c r="G38" s="850"/>
+      <c r="H38" s="851"/>
       <c r="I38" s="737"/>
       <c r="J38" s="715"/>
       <c r="K38" s="745"/>
@@ -15670,19 +15670,19 @@
       <c r="F39" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G39" s="830"/>
-      <c r="H39" s="831"/>
+      <c r="G39" s="850"/>
+      <c r="H39" s="851"/>
       <c r="I39" s="737"/>
       <c r="J39" s="715"/>
       <c r="K39" s="741"/>
       <c r="L39" s="737"/>
       <c r="M39" s="747"/>
       <c r="N39" s="121"/>
-      <c r="O39" s="832" t="s">
+      <c r="O39" s="831" t="s">
         <v>34</v>
       </c>
-      <c r="P39" s="832"/>
-      <c r="Q39" s="832"/>
+      <c r="P39" s="831"/>
+      <c r="Q39" s="831"/>
       <c r="R39" s="729"/>
       <c r="S39" s="729"/>
     </row>
@@ -15698,8 +15698,8 @@
       <c r="F40" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G40" s="830"/>
-      <c r="H40" s="831"/>
+      <c r="G40" s="850"/>
+      <c r="H40" s="851"/>
       <c r="I40" s="737"/>
       <c r="J40" s="715"/>
       <c r="K40" s="741"/>
@@ -15736,8 +15736,8 @@
       <c r="F41" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G41" s="830"/>
-      <c r="H41" s="831"/>
+      <c r="G41" s="850"/>
+      <c r="H41" s="851"/>
       <c r="I41" s="737"/>
       <c r="J41" s="715"/>
       <c r="K41" s="741"/>
@@ -15762,21 +15762,21 @@
       <c r="F42" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G42" s="830"/>
-      <c r="H42" s="831"/>
+      <c r="G42" s="850"/>
+      <c r="H42" s="851"/>
       <c r="I42" s="737"/>
       <c r="J42" s="715"/>
       <c r="K42" s="741"/>
       <c r="L42" s="737"/>
       <c r="M42" s="747"/>
       <c r="N42" s="121"/>
-      <c r="O42" s="833" t="s">
+      <c r="O42" s="874" t="s">
         <v>217</v>
       </c>
-      <c r="P42" s="834"/>
-      <c r="Q42" s="834"/>
-      <c r="R42" s="834"/>
-      <c r="S42" s="835"/>
+      <c r="P42" s="875"/>
+      <c r="Q42" s="875"/>
+      <c r="R42" s="875"/>
+      <c r="S42" s="876"/>
     </row>
     <row r="43" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="737" t="s">
@@ -15790,11 +15790,11 @@
       <c r="F43" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G43" s="828">
+      <c r="G43" s="852">
         <f>+G39-G41</f>
         <v>0</v>
       </c>
-      <c r="H43" s="829"/>
+      <c r="H43" s="853"/>
       <c r="I43" s="743">
         <f>+I39-I41</f>
         <v>0</v>
@@ -15813,15 +15813,15 @@
       </c>
       <c r="M43" s="747"/>
       <c r="N43" s="121"/>
-      <c r="O43" s="836" t="s">
+      <c r="O43" s="877" t="s">
         <v>212</v>
       </c>
-      <c r="P43" s="837"/>
-      <c r="Q43" s="836" t="s">
+      <c r="P43" s="878"/>
+      <c r="Q43" s="877" t="s">
         <v>213</v>
       </c>
-      <c r="R43" s="837"/>
-      <c r="S43" s="838" t="s">
+      <c r="R43" s="878"/>
+      <c r="S43" s="879" t="s">
         <v>214</v>
       </c>
     </row>
@@ -15837,11 +15837,11 @@
       <c r="F44" s="736" t="s">
         <v>109</v>
       </c>
-      <c r="G44" s="830">
+      <c r="G44" s="850">
         <f>+G41-G42</f>
         <v>0</v>
       </c>
-      <c r="H44" s="831"/>
+      <c r="H44" s="851"/>
       <c r="I44" s="737">
         <f>+I41-I42</f>
         <v>0</v>
@@ -15872,7 +15872,7 @@
       <c r="R44" s="750" t="s">
         <v>216</v>
       </c>
-      <c r="S44" s="839"/>
+      <c r="S44" s="880"/>
     </row>
     <row r="45" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="737" t="s">
@@ -15886,11 +15886,11 @@
       <c r="F45" s="736" t="s">
         <v>110</v>
       </c>
-      <c r="G45" s="828" t="e">
+      <c r="G45" s="852" t="e">
         <f>+G43/G44*100</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H45" s="829"/>
+      <c r="H45" s="853"/>
       <c r="I45" s="743" t="e">
         <f>+I43/I44*100</f>
         <v>#DIV/0!</v>
@@ -15943,15 +15943,15 @@
     </row>
     <row r="47" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="753"/>
-      <c r="B47" s="822" t="s">
+      <c r="B47" s="883" t="s">
         <v>308</v>
       </c>
-      <c r="C47" s="823"/>
-      <c r="D47" s="822" t="s">
+      <c r="C47" s="884"/>
+      <c r="D47" s="883" t="s">
         <v>309</v>
       </c>
-      <c r="E47" s="824"/>
-      <c r="F47" s="823"/>
+      <c r="E47" s="885"/>
+      <c r="F47" s="884"/>
       <c r="G47" s="754" t="s">
         <v>310</v>
       </c>
@@ -15967,9 +15967,9 @@
         <v>311</v>
       </c>
       <c r="C48" s="759"/>
-      <c r="D48" s="825"/>
-      <c r="E48" s="826"/>
-      <c r="F48" s="827"/>
+      <c r="D48" s="886"/>
+      <c r="E48" s="887"/>
+      <c r="F48" s="888"/>
       <c r="G48" s="760"/>
       <c r="H48" s="725"/>
       <c r="I48" s="725"/>
@@ -15983,9 +15983,9 @@
         <v>312</v>
       </c>
       <c r="C49" s="759"/>
-      <c r="D49" s="825"/>
-      <c r="E49" s="826"/>
-      <c r="F49" s="827"/>
+      <c r="D49" s="886"/>
+      <c r="E49" s="887"/>
+      <c r="F49" s="888"/>
       <c r="G49" s="762"/>
       <c r="N49" s="121"/>
     </row>
@@ -15994,9 +15994,9 @@
         <v>313</v>
       </c>
       <c r="C50" s="759"/>
-      <c r="D50" s="825"/>
-      <c r="E50" s="826"/>
-      <c r="F50" s="827"/>
+      <c r="D50" s="886"/>
+      <c r="E50" s="887"/>
+      <c r="F50" s="888"/>
       <c r="N50" s="121"/>
     </row>
     <row r="51" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -16004,17 +16004,17 @@
         <v>314</v>
       </c>
       <c r="C51" s="759"/>
-      <c r="D51" s="825"/>
-      <c r="E51" s="826"/>
-      <c r="F51" s="827"/>
+      <c r="D51" s="886"/>
+      <c r="E51" s="887"/>
+      <c r="F51" s="888"/>
       <c r="N51" s="121"/>
     </row>
     <row r="52" spans="1:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="763"/>
       <c r="C52" s="764"/>
-      <c r="D52" s="820"/>
-      <c r="E52" s="820"/>
-      <c r="F52" s="820"/>
+      <c r="D52" s="881"/>
+      <c r="E52" s="881"/>
+      <c r="F52" s="881"/>
       <c r="N52" s="121"/>
       <c r="O52" s="121"/>
     </row>
@@ -16060,21 +16060,21 @@
     </row>
     <row r="55" spans="1:15" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="821" t="s">
+      <c r="A56" s="882" t="s">
         <v>318</v>
       </c>
-      <c r="B56" s="821"/>
-      <c r="C56" s="821"/>
-      <c r="D56" s="821"/>
-      <c r="E56" s="821"/>
-      <c r="F56" s="821"/>
-      <c r="G56" s="821"/>
-      <c r="H56" s="821"/>
-      <c r="I56" s="821"/>
-      <c r="J56" s="821"/>
-      <c r="K56" s="821"/>
-      <c r="L56" s="821"/>
-      <c r="M56" s="821"/>
+      <c r="B56" s="882"/>
+      <c r="C56" s="882"/>
+      <c r="D56" s="882"/>
+      <c r="E56" s="882"/>
+      <c r="F56" s="882"/>
+      <c r="G56" s="882"/>
+      <c r="H56" s="882"/>
+      <c r="I56" s="882"/>
+      <c r="J56" s="882"/>
+      <c r="K56" s="882"/>
+      <c r="L56" s="882"/>
+      <c r="M56" s="882"/>
     </row>
     <row r="57" spans="1:15" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:15" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16085,43 +16085,14 @@
     <protectedRange sqref="C10:E11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="58">
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A7:M7"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="A13:M13"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="B16:L16"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="B24:L24"/>
-    <mergeCell ref="I26:L26"/>
-    <mergeCell ref="B28:L28"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="P37:Q37"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="J32:L32"/>
-    <mergeCell ref="J33:L33"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="B35:F36"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="A56:M56"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="D50:F50"/>
+    <mergeCell ref="D51:F51"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="G38:H38"/>
     <mergeCell ref="G39:H39"/>
@@ -16135,14 +16106,43 @@
     <mergeCell ref="Q43:R43"/>
     <mergeCell ref="S43:S44"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="A56:M56"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="B35:F36"/>
+    <mergeCell ref="G35:J35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="O36:Q36"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="P37:Q37"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="J32:L32"/>
+    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="I26:L26"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="A8:M8"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="A13:M13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -16194,43 +16194,43 @@
       <c r="N1" s="205"/>
     </row>
     <row r="2" spans="1:36" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="802" t="s">
+      <c r="A2" s="790" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="802"/>
-      <c r="C2" s="802"/>
-      <c r="D2" s="802"/>
-      <c r="E2" s="802"/>
-      <c r="F2" s="802"/>
-      <c r="G2" s="802"/>
-      <c r="H2" s="802"/>
-      <c r="I2" s="802"/>
-      <c r="J2" s="802"/>
-      <c r="K2" s="802"/>
-      <c r="L2" s="802"/>
-      <c r="M2" s="802"/>
-      <c r="N2" s="802"/>
+      <c r="B2" s="790"/>
+      <c r="C2" s="790"/>
+      <c r="D2" s="790"/>
+      <c r="E2" s="790"/>
+      <c r="F2" s="790"/>
+      <c r="G2" s="790"/>
+      <c r="H2" s="790"/>
+      <c r="I2" s="790"/>
+      <c r="J2" s="790"/>
+      <c r="K2" s="790"/>
+      <c r="L2" s="790"/>
+      <c r="M2" s="790"/>
+      <c r="N2" s="790"/>
       <c r="AJ2" s="180" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:36" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="902">
-        <v>0</v>
-      </c>
-      <c r="B3" s="902"/>
-      <c r="C3" s="902"/>
-      <c r="D3" s="902"/>
-      <c r="E3" s="902"/>
-      <c r="F3" s="902"/>
-      <c r="G3" s="902"/>
-      <c r="H3" s="902"/>
-      <c r="I3" s="902"/>
-      <c r="J3" s="902"/>
-      <c r="K3" s="902"/>
-      <c r="L3" s="902"/>
-      <c r="M3" s="902"/>
-      <c r="N3" s="902"/>
+      <c r="A3" s="899">
+        <v>0</v>
+      </c>
+      <c r="B3" s="899"/>
+      <c r="C3" s="899"/>
+      <c r="D3" s="899"/>
+      <c r="E3" s="899"/>
+      <c r="F3" s="899"/>
+      <c r="G3" s="899"/>
+      <c r="H3" s="899"/>
+      <c r="I3" s="899"/>
+      <c r="J3" s="899"/>
+      <c r="K3" s="899"/>
+      <c r="L3" s="899"/>
+      <c r="M3" s="899"/>
+      <c r="N3" s="899"/>
       <c r="AJ3" s="180" t="s">
         <v>145</v>
       </c>
@@ -16249,18 +16249,18 @@
       <c r="B5" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="906">
+      <c r="C5" s="903">
         <f>+FORMATO!Q2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="906"/>
-      <c r="E5" s="906"/>
-      <c r="F5" s="906"/>
-      <c r="G5" s="906"/>
-      <c r="H5" s="906"/>
-      <c r="I5" s="906"/>
-      <c r="J5" s="906"/>
-      <c r="K5" s="906"/>
+      <c r="D5" s="903"/>
+      <c r="E5" s="903"/>
+      <c r="F5" s="903"/>
+      <c r="G5" s="903"/>
+      <c r="H5" s="903"/>
+      <c r="I5" s="903"/>
+      <c r="J5" s="903"/>
+      <c r="K5" s="903"/>
       <c r="L5" s="30" t="s">
         <v>21</v>
       </c>
@@ -16278,17 +16278,17 @@
       <c r="B6" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="905">
+      <c r="C6" s="902">
         <f>+FORMATO!Q3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="905"/>
-      <c r="E6" s="905"/>
-      <c r="F6" s="905"/>
-      <c r="G6" s="905"/>
-      <c r="H6" s="905"/>
-      <c r="I6" s="905"/>
-      <c r="J6" s="905"/>
+      <c r="D6" s="902"/>
+      <c r="E6" s="902"/>
+      <c r="F6" s="902"/>
+      <c r="G6" s="902"/>
+      <c r="H6" s="902"/>
+      <c r="I6" s="902"/>
+      <c r="J6" s="902"/>
       <c r="K6" s="40"/>
       <c r="L6" s="34" t="s">
         <v>269</v>
@@ -16316,18 +16316,18 @@
       <c r="B7" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="906">
+      <c r="C7" s="903">
         <f>+FORMATO!Q4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="906"/>
-      <c r="E7" s="906"/>
-      <c r="F7" s="906"/>
-      <c r="G7" s="906"/>
-      <c r="H7" s="906"/>
-      <c r="I7" s="906"/>
-      <c r="J7" s="906"/>
-      <c r="K7" s="906"/>
+      <c r="D7" s="903"/>
+      <c r="E7" s="903"/>
+      <c r="F7" s="903"/>
+      <c r="G7" s="903"/>
+      <c r="H7" s="903"/>
+      <c r="I7" s="903"/>
+      <c r="J7" s="903"/>
+      <c r="K7" s="903"/>
       <c r="L7" s="34" t="s">
         <v>320</v>
       </c>
@@ -16359,17 +16359,17 @@
       <c r="B8" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="905">
+      <c r="C8" s="902">
         <f>+FORMATO!Q5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="905"/>
-      <c r="E8" s="905"/>
-      <c r="F8" s="905"/>
-      <c r="G8" s="905"/>
-      <c r="H8" s="905"/>
-      <c r="I8" s="905"/>
-      <c r="J8" s="905"/>
+      <c r="D8" s="902"/>
+      <c r="E8" s="902"/>
+      <c r="F8" s="902"/>
+      <c r="G8" s="902"/>
+      <c r="H8" s="902"/>
+      <c r="I8" s="902"/>
+      <c r="J8" s="902"/>
       <c r="K8" s="780"/>
       <c r="L8" s="34" t="s">
         <v>115</v>
@@ -16391,9 +16391,9 @@
       <c r="Y8" s="185"/>
       <c r="Z8" s="185"/>
       <c r="AA8" s="185"/>
-      <c r="AB8" s="907"/>
-      <c r="AC8" s="907"/>
-      <c r="AD8" s="907"/>
+      <c r="AB8" s="890"/>
+      <c r="AC8" s="890"/>
+      <c r="AD8" s="890"/>
     </row>
     <row r="9" spans="1:36" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="629" t="s">
@@ -16427,22 +16427,22 @@
       <c r="AD9" s="244"/>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A10" s="908" t="s">
+      <c r="A10" s="891" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="909"/>
-      <c r="C10" s="909"/>
-      <c r="D10" s="909"/>
-      <c r="E10" s="909"/>
-      <c r="F10" s="909"/>
-      <c r="G10" s="909"/>
-      <c r="H10" s="909"/>
-      <c r="I10" s="909"/>
-      <c r="J10" s="909"/>
-      <c r="K10" s="909"/>
-      <c r="L10" s="909"/>
-      <c r="M10" s="909"/>
-      <c r="N10" s="910"/>
+      <c r="B10" s="892"/>
+      <c r="C10" s="892"/>
+      <c r="D10" s="892"/>
+      <c r="E10" s="892"/>
+      <c r="F10" s="892"/>
+      <c r="G10" s="892"/>
+      <c r="H10" s="892"/>
+      <c r="I10" s="892"/>
+      <c r="J10" s="892"/>
+      <c r="K10" s="892"/>
+      <c r="L10" s="892"/>
+      <c r="M10" s="892"/>
+      <c r="N10" s="893"/>
       <c r="O10" s="183"/>
       <c r="P10" s="183"/>
       <c r="Q10" s="183"/>
@@ -16458,22 +16458,22 @@
       <c r="AD10" s="244"/>
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A11" s="911" t="s">
+      <c r="A11" s="894" t="s">
         <v>236</v>
       </c>
-      <c r="B11" s="912"/>
-      <c r="C11" s="912"/>
-      <c r="D11" s="912"/>
-      <c r="E11" s="912"/>
-      <c r="F11" s="912"/>
-      <c r="G11" s="912"/>
-      <c r="H11" s="912"/>
-      <c r="I11" s="912"/>
-      <c r="J11" s="912"/>
-      <c r="K11" s="912"/>
-      <c r="L11" s="912"/>
-      <c r="M11" s="912"/>
-      <c r="N11" s="913"/>
+      <c r="B11" s="895"/>
+      <c r="C11" s="895"/>
+      <c r="D11" s="895"/>
+      <c r="E11" s="895"/>
+      <c r="F11" s="895"/>
+      <c r="G11" s="895"/>
+      <c r="H11" s="895"/>
+      <c r="I11" s="895"/>
+      <c r="J11" s="895"/>
+      <c r="K11" s="895"/>
+      <c r="L11" s="895"/>
+      <c r="M11" s="895"/>
+      <c r="N11" s="896"/>
       <c r="O11" s="183"/>
       <c r="P11" s="183"/>
       <c r="Q11" s="183"/>
@@ -16750,8 +16750,8 @@
       <c r="I19" s="211"/>
       <c r="J19" s="211"/>
       <c r="K19" s="211"/>
-      <c r="L19" s="803"/>
-      <c r="M19" s="803"/>
+      <c r="L19" s="791"/>
+      <c r="M19" s="791"/>
       <c r="N19" s="53"/>
       <c r="O19" s="183"/>
       <c r="P19" s="198"/>
@@ -16759,18 +16759,18 @@
       <c r="R19" s="198"/>
       <c r="S19" s="198"/>
       <c r="T19" s="198"/>
-      <c r="U19" s="890" t="s">
+      <c r="U19" s="889" t="s">
         <v>197</v>
       </c>
-      <c r="V19" s="915" t="s">
+      <c r="V19" s="898" t="s">
         <v>35</v>
       </c>
-      <c r="W19" s="915"/>
-      <c r="X19" s="915"/>
-      <c r="Y19" s="915" t="s">
+      <c r="W19" s="898"/>
+      <c r="X19" s="898"/>
+      <c r="Y19" s="898" t="s">
         <v>34</v>
       </c>
-      <c r="Z19" s="915"/>
+      <c r="Z19" s="898"/>
       <c r="AA19" s="199"/>
       <c r="AB19" s="199"/>
       <c r="AC19" s="199"/>
@@ -16779,27 +16779,27 @@
       <c r="AF19" s="199"/>
     </row>
     <row r="20" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="805" t="s">
+      <c r="A20" s="793" t="s">
         <v>146</v>
       </c>
-      <c r="B20" s="806"/>
-      <c r="C20" s="806"/>
-      <c r="D20" s="806"/>
-      <c r="E20" s="806"/>
+      <c r="B20" s="794"/>
+      <c r="C20" s="794"/>
+      <c r="D20" s="794"/>
+      <c r="E20" s="794"/>
       <c r="F20" s="212" t="s">
         <v>113</v>
       </c>
-      <c r="G20" s="805" t="s">
+      <c r="G20" s="793" t="s">
         <v>206</v>
       </c>
-      <c r="H20" s="806"/>
-      <c r="I20" s="903"/>
-      <c r="J20" s="904" t="s">
+      <c r="H20" s="794"/>
+      <c r="I20" s="900"/>
+      <c r="J20" s="901" t="s">
         <v>205</v>
       </c>
-      <c r="K20" s="808"/>
-      <c r="L20" s="804"/>
-      <c r="M20" s="804"/>
+      <c r="K20" s="796"/>
+      <c r="L20" s="792"/>
+      <c r="M20" s="792"/>
       <c r="N20" s="57"/>
       <c r="O20" s="183"/>
       <c r="P20" s="200"/>
@@ -16807,18 +16807,18 @@
       <c r="R20" s="200"/>
       <c r="S20" s="200"/>
       <c r="T20" s="200"/>
-      <c r="U20" s="890"/>
-      <c r="V20" s="914" t="str">
+      <c r="U20" s="889"/>
+      <c r="V20" s="897" t="str">
         <f>+DATOS!C12</f>
         <v>-</v>
       </c>
-      <c r="W20" s="914"/>
-      <c r="X20" s="914"/>
-      <c r="Y20" s="914" t="str">
+      <c r="W20" s="897"/>
+      <c r="X20" s="897"/>
+      <c r="Y20" s="897" t="str">
         <f>+DATOS!I12</f>
         <v>-</v>
       </c>
-      <c r="Z20" s="914"/>
+      <c r="Z20" s="897"/>
       <c r="AA20" s="199"/>
       <c r="AB20" s="199"/>
       <c r="AC20" s="199"/>
@@ -16827,13 +16827,13 @@
       <c r="AF20" s="199"/>
     </row>
     <row r="21" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="793" t="s">
+      <c r="A21" s="808" t="s">
         <v>147</v>
       </c>
-      <c r="B21" s="794"/>
-      <c r="C21" s="794"/>
-      <c r="D21" s="794"/>
-      <c r="E21" s="795"/>
+      <c r="B21" s="809"/>
+      <c r="C21" s="809"/>
+      <c r="D21" s="809"/>
+      <c r="E21" s="810"/>
       <c r="F21" s="213" t="s">
         <v>148</v>
       </c>
@@ -16857,8 +16857,8 @@
         <f>IF($Y$20="NO",Z21,IF($Y$20="-","",Z21))</f>
         <v/>
       </c>
-      <c r="L21" s="804"/>
-      <c r="M21" s="804"/>
+      <c r="L21" s="792"/>
+      <c r="M21" s="792"/>
       <c r="N21" s="57"/>
       <c r="O21" s="183"/>
       <c r="P21" s="200"/>
@@ -16892,13 +16892,13 @@
       <c r="AF21" s="199"/>
     </row>
     <row r="22" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="790" t="s">
+      <c r="A22" s="787" t="s">
         <v>149</v>
       </c>
-      <c r="B22" s="791"/>
-      <c r="C22" s="791"/>
-      <c r="D22" s="791"/>
-      <c r="E22" s="792"/>
+      <c r="B22" s="788"/>
+      <c r="C22" s="788"/>
+      <c r="D22" s="788"/>
+      <c r="E22" s="789"/>
       <c r="F22" s="213" t="s">
         <v>148</v>
       </c>
@@ -16922,8 +16922,8 @@
         <f>IF($Y$20="NO","--",IF($Y$20="-","",Z22))</f>
         <v/>
       </c>
-      <c r="L22" s="813"/>
-      <c r="M22" s="813"/>
+      <c r="L22" s="801"/>
+      <c r="M22" s="801"/>
       <c r="N22" s="69"/>
       <c r="O22" s="201"/>
       <c r="P22" s="200"/>
@@ -16962,13 +16962,13 @@
       <c r="AF22" s="199"/>
     </row>
     <row r="23" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="790" t="s">
+      <c r="A23" s="787" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="791"/>
-      <c r="C23" s="791"/>
-      <c r="D23" s="791"/>
-      <c r="E23" s="792"/>
+      <c r="B23" s="788"/>
+      <c r="C23" s="788"/>
+      <c r="D23" s="788"/>
+      <c r="E23" s="789"/>
       <c r="F23" s="213" t="s">
         <v>148</v>
       </c>
@@ -17024,13 +17024,13 @@
       <c r="AF23" s="199"/>
     </row>
     <row r="24" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="790" t="s">
+      <c r="A24" s="787" t="s">
         <v>208</v>
       </c>
-      <c r="B24" s="791"/>
-      <c r="C24" s="791"/>
-      <c r="D24" s="791"/>
-      <c r="E24" s="792"/>
+      <c r="B24" s="788"/>
+      <c r="C24" s="788"/>
+      <c r="D24" s="788"/>
+      <c r="E24" s="789"/>
       <c r="F24" s="213" t="s">
         <v>109</v>
       </c>
@@ -17094,13 +17094,13 @@
       <c r="AF24" s="199"/>
     </row>
     <row r="25" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="790" t="s">
+      <c r="A25" s="787" t="s">
         <v>209</v>
       </c>
-      <c r="B25" s="791"/>
-      <c r="C25" s="791"/>
-      <c r="D25" s="791"/>
-      <c r="E25" s="792"/>
+      <c r="B25" s="788"/>
+      <c r="C25" s="788"/>
+      <c r="D25" s="788"/>
+      <c r="E25" s="789"/>
       <c r="F25" s="213" t="s">
         <v>109</v>
       </c>
@@ -17164,13 +17164,13 @@
       <c r="AF25" s="199"/>
     </row>
     <row r="26" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="790" t="s">
+      <c r="A26" s="787" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="791"/>
-      <c r="C26" s="791"/>
-      <c r="D26" s="791"/>
-      <c r="E26" s="792"/>
+      <c r="B26" s="788"/>
+      <c r="C26" s="788"/>
+      <c r="D26" s="788"/>
+      <c r="E26" s="789"/>
       <c r="F26" s="213" t="s">
         <v>109</v>
       </c>
@@ -17234,13 +17234,13 @@
       <c r="AF26" s="199"/>
     </row>
     <row r="27" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="790" t="s">
+      <c r="A27" s="787" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="791"/>
-      <c r="C27" s="791"/>
-      <c r="D27" s="791"/>
-      <c r="E27" s="792"/>
+      <c r="B27" s="788"/>
+      <c r="C27" s="788"/>
+      <c r="D27" s="788"/>
+      <c r="E27" s="789"/>
       <c r="F27" s="213" t="s">
         <v>109</v>
       </c>
@@ -17304,13 +17304,13 @@
       <c r="AF27" s="199"/>
     </row>
     <row r="28" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="790" t="s">
+      <c r="A28" s="787" t="s">
         <v>210</v>
       </c>
-      <c r="B28" s="791"/>
-      <c r="C28" s="791"/>
-      <c r="D28" s="791"/>
-      <c r="E28" s="792"/>
+      <c r="B28" s="788"/>
+      <c r="C28" s="788"/>
+      <c r="D28" s="788"/>
+      <c r="E28" s="789"/>
       <c r="F28" s="213" t="s">
         <v>109</v>
       </c>
@@ -17374,13 +17374,13 @@
       <c r="AF28" s="199"/>
     </row>
     <row r="29" spans="1:32" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="793" t="s">
+      <c r="A29" s="808" t="s">
         <v>111</v>
       </c>
-      <c r="B29" s="794"/>
-      <c r="C29" s="794"/>
-      <c r="D29" s="794"/>
-      <c r="E29" s="795"/>
+      <c r="B29" s="809"/>
+      <c r="C29" s="809"/>
+      <c r="D29" s="809"/>
+      <c r="E29" s="810"/>
       <c r="F29" s="217" t="s">
         <v>110</v>
       </c>
@@ -17521,11 +17521,11 @@
       <c r="V31" s="180"/>
       <c r="W31" s="233"/>
       <c r="X31" s="261"/>
-      <c r="Y31" s="901" t="e">
+      <c r="Y31" s="904" t="e">
         <f>AVERAGE(Y30:Z30)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z31" s="901"/>
+      <c r="Z31" s="904"/>
       <c r="AA31" s="199"/>
       <c r="AB31" s="199"/>
       <c r="AC31" s="199"/>
@@ -17543,10 +17543,10 @@
       <c r="G32" s="21"/>
       <c r="H32" s="21"/>
       <c r="I32" s="21"/>
-      <c r="J32" s="781" t="s">
+      <c r="J32" s="811" t="s">
         <v>203</v>
       </c>
-      <c r="K32" s="782"/>
+      <c r="K32" s="812"/>
       <c r="L32" s="221" t="str">
         <f>IF(V20="-","",IF(V20="NO","NP",ROUND(V42,0)))</f>
         <v/>
@@ -17620,10 +17620,10 @@
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
       <c r="I34" s="21"/>
-      <c r="J34" s="781" t="s">
+      <c r="J34" s="811" t="s">
         <v>204</v>
       </c>
-      <c r="K34" s="782"/>
+      <c r="K34" s="812"/>
       <c r="L34" s="221" t="str">
         <f>IF(V20="-","",IF(Y20="NO","NP",ROUND(Y31,0)))</f>
         <v/>
@@ -17717,10 +17717,10 @@
       <c r="G36" s="209"/>
       <c r="H36" s="209"/>
       <c r="I36" s="209"/>
-      <c r="J36" s="781" t="s">
+      <c r="J36" s="811" t="s">
         <v>77</v>
       </c>
-      <c r="K36" s="782"/>
+      <c r="K36" s="812"/>
       <c r="L36" s="221" t="str">
         <f>IF(Y20="-","",IF(Y20="NO","NP",L32-L34))</f>
         <v/>
@@ -17970,10 +17970,10 @@
       </c>
       <c r="V42" s="598"/>
       <c r="W42" s="525"/>
-      <c r="X42" s="892" t="s">
+      <c r="X42" s="905" t="s">
         <v>175</v>
       </c>
-      <c r="Y42" s="893"/>
+      <c r="Y42" s="906"/>
       <c r="Z42" s="577" t="e">
         <f>(Z39*LN(25)+Z40)</f>
         <v>#VALUE!</v>
@@ -18263,13 +18263,13 @@
       <c r="H52" s="293"/>
       <c r="I52" s="231"/>
       <c r="J52" s="231"/>
-      <c r="K52" s="890">
+      <c r="K52" s="889">
         <f>+FORMATO!J17</f>
         <v>0</v>
       </c>
-      <c r="L52" s="890"/>
-      <c r="M52" s="890"/>
-      <c r="N52" s="890"/>
+      <c r="L52" s="889"/>
+      <c r="M52" s="889"/>
+      <c r="N52" s="889"/>
       <c r="O52" s="203"/>
       <c r="P52" s="183"/>
       <c r="Q52" s="183"/>
@@ -18290,13 +18290,13 @@
       <c r="H53" s="293"/>
       <c r="I53" s="231"/>
       <c r="J53" s="231"/>
-      <c r="K53" s="890">
+      <c r="K53" s="889">
         <f>+FORMATO!J18</f>
         <v>0</v>
       </c>
-      <c r="L53" s="890"/>
-      <c r="M53" s="890"/>
-      <c r="N53" s="890"/>
+      <c r="L53" s="889"/>
+      <c r="M53" s="889"/>
+      <c r="N53" s="889"/>
       <c r="O53" s="203"/>
       <c r="P53" s="183"/>
       <c r="Q53" s="183"/>
@@ -18317,13 +18317,13 @@
       <c r="H54" s="293"/>
       <c r="I54" s="231"/>
       <c r="J54" s="231"/>
-      <c r="K54" s="890">
+      <c r="K54" s="889">
         <f>+FORMATO!J19</f>
         <v>0</v>
       </c>
-      <c r="L54" s="890"/>
-      <c r="M54" s="890"/>
-      <c r="N54" s="890"/>
+      <c r="L54" s="889"/>
+      <c r="M54" s="889"/>
+      <c r="N54" s="889"/>
       <c r="O54" s="203"/>
       <c r="P54" s="183"/>
       <c r="Q54" s="183"/>
@@ -18344,13 +18344,13 @@
       <c r="H55" s="293"/>
       <c r="I55" s="231"/>
       <c r="J55" s="231"/>
-      <c r="K55" s="890">
+      <c r="K55" s="889">
         <f>+FORMATO!J20</f>
         <v>0</v>
       </c>
-      <c r="L55" s="890"/>
-      <c r="M55" s="890"/>
-      <c r="N55" s="890"/>
+      <c r="L55" s="889"/>
+      <c r="M55" s="889"/>
+      <c r="N55" s="889"/>
       <c r="O55" s="203"/>
       <c r="P55" s="183"/>
       <c r="Q55" s="183"/>
@@ -18372,13 +18372,13 @@
       <c r="H56" s="293"/>
       <c r="I56" s="231"/>
       <c r="J56" s="231"/>
-      <c r="K56" s="890">
+      <c r="K56" s="889">
         <f>+FORMATO!J22</f>
         <v>0</v>
       </c>
-      <c r="L56" s="890"/>
-      <c r="M56" s="890"/>
-      <c r="N56" s="890"/>
+      <c r="L56" s="889"/>
+      <c r="M56" s="889"/>
+      <c r="N56" s="889"/>
       <c r="O56" s="203"/>
       <c r="P56" s="183"/>
       <c r="Q56" s="183"/>
@@ -18399,13 +18399,13 @@
       <c r="H57" s="231"/>
       <c r="I57" s="231"/>
       <c r="J57" s="231"/>
-      <c r="K57" s="890">
+      <c r="K57" s="889">
         <f>+FORMATO!J23</f>
         <v>0</v>
       </c>
-      <c r="L57" s="890"/>
-      <c r="M57" s="890"/>
-      <c r="N57" s="890"/>
+      <c r="L57" s="889"/>
+      <c r="M57" s="889"/>
+      <c r="N57" s="889"/>
       <c r="O57" s="290"/>
       <c r="P57" s="183"/>
       <c r="Q57" s="183"/>
@@ -18469,11 +18469,11 @@
       <c r="F60" s="179"/>
       <c r="G60" s="179"/>
       <c r="H60" s="179"/>
-      <c r="I60" s="890">
+      <c r="I60" s="889">
         <f>+FORMATO!J29</f>
         <v>0</v>
       </c>
-      <c r="J60" s="890"/>
+      <c r="J60" s="889"/>
       <c r="K60" s="231"/>
       <c r="L60" s="231"/>
       <c r="M60" s="231"/>
@@ -18495,11 +18495,11 @@
       <c r="F61" s="179"/>
       <c r="G61" s="179"/>
       <c r="H61" s="179"/>
-      <c r="I61" s="890">
+      <c r="I61" s="889">
         <f>+FORMATO!J30</f>
         <v>0</v>
       </c>
-      <c r="J61" s="890"/>
+      <c r="J61" s="889"/>
       <c r="K61" s="231"/>
       <c r="L61" s="231"/>
       <c r="M61" s="231"/>
@@ -18521,11 +18521,11 @@
       <c r="F62" s="179"/>
       <c r="G62" s="179"/>
       <c r="H62" s="179"/>
-      <c r="I62" s="890">
+      <c r="I62" s="889">
         <f>+FORMATO!J31</f>
         <v>0</v>
       </c>
-      <c r="J62" s="890"/>
+      <c r="J62" s="889"/>
       <c r="K62" s="231"/>
       <c r="L62" s="231"/>
       <c r="M62" s="231"/>
@@ -18547,11 +18547,11 @@
       <c r="F63" s="179"/>
       <c r="G63" s="179"/>
       <c r="H63" s="179"/>
-      <c r="I63" s="895">
+      <c r="I63" s="909">
         <f>+FORMATO!J32</f>
         <v>0</v>
       </c>
-      <c r="J63" s="895"/>
+      <c r="J63" s="909"/>
       <c r="K63" s="231"/>
       <c r="L63" s="231"/>
       <c r="M63" s="231"/>
@@ -18573,11 +18573,11 @@
       <c r="F64" s="179"/>
       <c r="G64" s="179"/>
       <c r="H64" s="179"/>
-      <c r="I64" s="890">
+      <c r="I64" s="889">
         <f>+FORMATO!J33</f>
         <v>0</v>
       </c>
-      <c r="J64" s="890"/>
+      <c r="J64" s="889"/>
       <c r="K64" s="231"/>
       <c r="L64" s="231"/>
       <c r="M64" s="231"/>
@@ -18599,17 +18599,17 @@
       <c r="F65" s="301"/>
       <c r="G65" s="301"/>
       <c r="H65" s="301"/>
-      <c r="I65" s="896">
+      <c r="I65" s="910">
         <f>+FORMATO!J21</f>
         <v>0</v>
       </c>
-      <c r="J65" s="896"/>
-      <c r="K65" s="898">
-        <v>0</v>
-      </c>
-      <c r="L65" s="899"/>
-      <c r="M65" s="899"/>
-      <c r="N65" s="899"/>
+      <c r="J65" s="910"/>
+      <c r="K65" s="912">
+        <v>0</v>
+      </c>
+      <c r="L65" s="913"/>
+      <c r="M65" s="913"/>
+      <c r="N65" s="913"/>
       <c r="O65" s="296"/>
       <c r="P65" s="183"/>
       <c r="Q65" s="179"/>
@@ -18652,94 +18652,94 @@
       <c r="N67" s="178"/>
     </row>
     <row r="68" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="900" t="s">
+      <c r="A68" s="914" t="s">
         <v>337</v>
       </c>
-      <c r="B68" s="900"/>
-      <c r="C68" s="900"/>
-      <c r="D68" s="900"/>
-      <c r="E68" s="900"/>
-      <c r="F68" s="900"/>
-      <c r="G68" s="900"/>
-      <c r="H68" s="900"/>
-      <c r="I68" s="900"/>
-      <c r="J68" s="900"/>
-      <c r="K68" s="900"/>
-      <c r="L68" s="900"/>
-      <c r="M68" s="900"/>
-      <c r="N68" s="900"/>
+      <c r="B68" s="914"/>
+      <c r="C68" s="914"/>
+      <c r="D68" s="914"/>
+      <c r="E68" s="914"/>
+      <c r="F68" s="914"/>
+      <c r="G68" s="914"/>
+      <c r="H68" s="914"/>
+      <c r="I68" s="914"/>
+      <c r="J68" s="914"/>
+      <c r="K68" s="914"/>
+      <c r="L68" s="914"/>
+      <c r="M68" s="914"/>
+      <c r="N68" s="914"/>
     </row>
     <row r="69" spans="1:19" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="897" t="s">
+      <c r="A69" s="911" t="s">
         <v>338</v>
       </c>
-      <c r="B69" s="897"/>
-      <c r="C69" s="897"/>
-      <c r="D69" s="897"/>
-      <c r="E69" s="897"/>
-      <c r="F69" s="897"/>
-      <c r="G69" s="897"/>
-      <c r="H69" s="897"/>
-      <c r="I69" s="897"/>
-      <c r="J69" s="897"/>
-      <c r="K69" s="897"/>
-      <c r="L69" s="897"/>
-      <c r="M69" s="897"/>
-      <c r="N69" s="897"/>
+      <c r="B69" s="911"/>
+      <c r="C69" s="911"/>
+      <c r="D69" s="911"/>
+      <c r="E69" s="911"/>
+      <c r="F69" s="911"/>
+      <c r="G69" s="911"/>
+      <c r="H69" s="911"/>
+      <c r="I69" s="911"/>
+      <c r="J69" s="911"/>
+      <c r="K69" s="911"/>
+      <c r="L69" s="911"/>
+      <c r="M69" s="911"/>
+      <c r="N69" s="911"/>
     </row>
     <row r="70" spans="1:19" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="897" t="s">
+      <c r="A70" s="911" t="s">
         <v>339</v>
       </c>
-      <c r="B70" s="897"/>
-      <c r="C70" s="897"/>
-      <c r="D70" s="897"/>
-      <c r="E70" s="897"/>
-      <c r="F70" s="897"/>
-      <c r="G70" s="897"/>
-      <c r="H70" s="897"/>
-      <c r="I70" s="897"/>
-      <c r="J70" s="897"/>
-      <c r="K70" s="897"/>
-      <c r="L70" s="897"/>
-      <c r="M70" s="897"/>
-      <c r="N70" s="897"/>
+      <c r="B70" s="911"/>
+      <c r="C70" s="911"/>
+      <c r="D70" s="911"/>
+      <c r="E70" s="911"/>
+      <c r="F70" s="911"/>
+      <c r="G70" s="911"/>
+      <c r="H70" s="911"/>
+      <c r="I70" s="911"/>
+      <c r="J70" s="911"/>
+      <c r="K70" s="911"/>
+      <c r="L70" s="911"/>
+      <c r="M70" s="911"/>
+      <c r="N70" s="911"/>
     </row>
     <row r="71" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="897" t="s">
+      <c r="A71" s="911" t="s">
         <v>340</v>
       </c>
-      <c r="B71" s="897"/>
-      <c r="C71" s="897"/>
-      <c r="D71" s="897"/>
-      <c r="E71" s="897"/>
-      <c r="F71" s="897"/>
-      <c r="G71" s="897"/>
-      <c r="H71" s="897"/>
-      <c r="I71" s="897"/>
-      <c r="J71" s="897"/>
-      <c r="K71" s="897"/>
-      <c r="L71" s="897"/>
-      <c r="M71" s="897"/>
-      <c r="N71" s="897"/>
+      <c r="B71" s="911"/>
+      <c r="C71" s="911"/>
+      <c r="D71" s="911"/>
+      <c r="E71" s="911"/>
+      <c r="F71" s="911"/>
+      <c r="G71" s="911"/>
+      <c r="H71" s="911"/>
+      <c r="I71" s="911"/>
+      <c r="J71" s="911"/>
+      <c r="K71" s="911"/>
+      <c r="L71" s="911"/>
+      <c r="M71" s="911"/>
+      <c r="N71" s="911"/>
     </row>
     <row r="72" spans="1:19" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="894" t="s">
+      <c r="A72" s="908" t="s">
         <v>341</v>
       </c>
-      <c r="B72" s="894"/>
-      <c r="C72" s="894"/>
-      <c r="D72" s="894"/>
-      <c r="E72" s="894"/>
-      <c r="F72" s="894"/>
-      <c r="G72" s="894"/>
-      <c r="H72" s="894"/>
-      <c r="I72" s="894"/>
-      <c r="J72" s="894"/>
-      <c r="K72" s="894"/>
-      <c r="L72" s="894"/>
-      <c r="M72" s="894"/>
-      <c r="N72" s="894"/>
+      <c r="B72" s="908"/>
+      <c r="C72" s="908"/>
+      <c r="D72" s="908"/>
+      <c r="E72" s="908"/>
+      <c r="F72" s="908"/>
+      <c r="G72" s="908"/>
+      <c r="H72" s="908"/>
+      <c r="I72" s="908"/>
+      <c r="J72" s="908"/>
+      <c r="K72" s="908"/>
+      <c r="L72" s="908"/>
+      <c r="M72" s="908"/>
+      <c r="N72" s="908"/>
     </row>
     <row r="73" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="294"/>
@@ -18784,10 +18784,10 @@
       <c r="A76" s="294"/>
       <c r="B76" s="294"/>
       <c r="C76" s="294"/>
-      <c r="K76" s="889"/>
-      <c r="L76" s="889"/>
-      <c r="M76" s="889"/>
-      <c r="N76" s="889"/>
+      <c r="K76" s="907"/>
+      <c r="L76" s="907"/>
+      <c r="M76" s="907"/>
+      <c r="N76" s="907"/>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="294"/>
@@ -18862,20 +18862,20 @@
       <c r="N84" s="295"/>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A85" s="891"/>
-      <c r="B85" s="891"/>
-      <c r="C85" s="891"/>
-      <c r="D85" s="891"/>
-      <c r="E85" s="891"/>
-      <c r="F85" s="891"/>
-      <c r="G85" s="891"/>
-      <c r="H85" s="891"/>
-      <c r="I85" s="891"/>
-      <c r="J85" s="891"/>
-      <c r="K85" s="891"/>
-      <c r="L85" s="891"/>
-      <c r="M85" s="891"/>
-      <c r="N85" s="891"/>
+      <c r="A85" s="915"/>
+      <c r="B85" s="915"/>
+      <c r="C85" s="915"/>
+      <c r="D85" s="915"/>
+      <c r="E85" s="915"/>
+      <c r="F85" s="915"/>
+      <c r="G85" s="915"/>
+      <c r="H85" s="915"/>
+      <c r="I85" s="915"/>
+      <c r="J85" s="915"/>
+      <c r="K85" s="915"/>
+      <c r="L85" s="915"/>
+      <c r="M85" s="915"/>
+      <c r="N85" s="915"/>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="92" t="s">
@@ -18890,10 +18890,10 @@
       <c r="H86" s="205"/>
       <c r="I86" s="205"/>
       <c r="J86" s="205"/>
-      <c r="K86" s="889"/>
-      <c r="L86" s="889"/>
-      <c r="M86" s="889"/>
-      <c r="N86" s="889"/>
+      <c r="K86" s="907"/>
+      <c r="L86" s="907"/>
+      <c r="M86" s="907"/>
+      <c r="N86" s="907"/>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="92" t="s">
@@ -18908,12 +18908,12 @@
       <c r="H87" s="205"/>
       <c r="I87" s="205"/>
       <c r="J87" s="205"/>
-      <c r="K87" s="889" t="s">
+      <c r="K87" s="907" t="s">
         <v>220</v>
       </c>
-      <c r="L87" s="889"/>
-      <c r="M87" s="889"/>
-      <c r="N87" s="889"/>
+      <c r="L87" s="907"/>
+      <c r="M87" s="907"/>
+      <c r="N87" s="907"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="205"/>
@@ -18986,42 +18986,12 @@
     <protectedRange sqref="E5:F6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="57">
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="K52:N52"/>
-    <mergeCell ref="K53:N53"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="AB8:AD8"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="V20:X20"/>
-    <mergeCell ref="Y20:Z20"/>
-    <mergeCell ref="Y19:Z19"/>
-    <mergeCell ref="V19:X19"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="K87:N87"/>
+    <mergeCell ref="K54:N54"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="K86:N86"/>
+    <mergeCell ref="A85:N85"/>
     <mergeCell ref="X42:Y42"/>
     <mergeCell ref="K76:N76"/>
     <mergeCell ref="I64:J64"/>
@@ -19037,12 +19007,42 @@
     <mergeCell ref="A68:N68"/>
     <mergeCell ref="A69:N69"/>
     <mergeCell ref="A71:N71"/>
-    <mergeCell ref="K87:N87"/>
-    <mergeCell ref="K54:N54"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="K86:N86"/>
-    <mergeCell ref="A85:N85"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="AB8:AD8"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="A11:N11"/>
+    <mergeCell ref="V20:X20"/>
+    <mergeCell ref="Y20:Z20"/>
+    <mergeCell ref="Y19:Z19"/>
+    <mergeCell ref="V19:X19"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="K52:N52"/>
+    <mergeCell ref="K53:N53"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.98425196850393704" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -19072,34 +19072,34 @@
   <sheetData>
     <row r="1" spans="1:12" ht="7.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="922" t="s">
+      <c r="B2" s="928" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="922"/>
-      <c r="D2" s="922"/>
-      <c r="E2" s="922"/>
-      <c r="F2" s="922"/>
-      <c r="G2" s="922"/>
-      <c r="H2" s="922"/>
-      <c r="I2" s="922"/>
-      <c r="J2" s="922"/>
-      <c r="K2" s="922"/>
-      <c r="L2" s="922"/>
+      <c r="C2" s="928"/>
+      <c r="D2" s="928"/>
+      <c r="E2" s="928"/>
+      <c r="F2" s="928"/>
+      <c r="G2" s="928"/>
+      <c r="H2" s="928"/>
+      <c r="I2" s="928"/>
+      <c r="J2" s="928"/>
+      <c r="K2" s="928"/>
+      <c r="L2" s="928"/>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="922" t="s">
+      <c r="B3" s="928" t="s">
         <v>236</v>
       </c>
-      <c r="C3" s="922"/>
-      <c r="D3" s="922"/>
-      <c r="E3" s="922"/>
-      <c r="F3" s="922"/>
-      <c r="G3" s="922"/>
-      <c r="H3" s="922"/>
-      <c r="I3" s="922"/>
-      <c r="J3" s="922"/>
-      <c r="K3" s="922"/>
-      <c r="L3" s="922"/>
+      <c r="C3" s="928"/>
+      <c r="D3" s="928"/>
+      <c r="E3" s="928"/>
+      <c r="F3" s="928"/>
+      <c r="G3" s="928"/>
+      <c r="H3" s="928"/>
+      <c r="I3" s="928"/>
+      <c r="J3" s="928"/>
+      <c r="K3" s="928"/>
+      <c r="L3" s="928"/>
     </row>
     <row r="4" spans="1:12" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="311"/>
@@ -19211,45 +19211,45 @@
     </row>
     <row r="11" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="255"/>
-      <c r="B11" s="921" t="s">
+      <c r="B11" s="927" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="808" t="s">
+      <c r="C11" s="796" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="808"/>
-      <c r="E11" s="808"/>
-      <c r="F11" s="808"/>
-      <c r="G11" s="808"/>
-      <c r="H11" s="808"/>
-      <c r="I11" s="808" t="s">
+      <c r="D11" s="796"/>
+      <c r="E11" s="796"/>
+      <c r="F11" s="796"/>
+      <c r="G11" s="796"/>
+      <c r="H11" s="796"/>
+      <c r="I11" s="796" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="808"/>
-      <c r="K11" s="808"/>
-      <c r="L11" s="808"/>
+      <c r="J11" s="796"/>
+      <c r="K11" s="796"/>
+      <c r="L11" s="796"/>
     </row>
     <row r="12" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="255"/>
-      <c r="B12" s="921"/>
-      <c r="C12" s="927" t="s">
+      <c r="B12" s="927"/>
+      <c r="C12" s="919" t="s">
         <v>198</v>
       </c>
-      <c r="D12" s="927"/>
-      <c r="E12" s="927"/>
-      <c r="F12" s="927"/>
-      <c r="G12" s="927"/>
-      <c r="H12" s="927"/>
-      <c r="I12" s="927" t="s">
+      <c r="D12" s="919"/>
+      <c r="E12" s="919"/>
+      <c r="F12" s="919"/>
+      <c r="G12" s="919"/>
+      <c r="H12" s="919"/>
+      <c r="I12" s="919" t="s">
         <v>198</v>
       </c>
-      <c r="J12" s="927"/>
-      <c r="K12" s="927"/>
-      <c r="L12" s="927"/>
+      <c r="J12" s="919"/>
+      <c r="K12" s="919"/>
+      <c r="L12" s="919"/>
     </row>
     <row r="13" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="255"/>
-      <c r="B13" s="921"/>
+      <c r="B13" s="927"/>
       <c r="C13" s="250" t="s">
         <v>196</v>
       </c>
@@ -19747,13 +19747,13 @@
       <c r="F24" s="83"/>
       <c r="G24" s="83"/>
       <c r="H24" s="83"/>
-      <c r="I24" s="923" t="e">
+      <c r="I24" s="929" t="e">
         <f>+AVERAGE(J23,L23)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="923"/>
-      <c r="K24" s="923"/>
-      <c r="L24" s="923"/>
+      <c r="J24" s="929"/>
+      <c r="K24" s="929"/>
+      <c r="L24" s="929"/>
       <c r="N24" s="264"/>
       <c r="O24" s="263"/>
       <c r="P24" s="263"/>
@@ -19873,13 +19873,13 @@
       </c>
       <c r="G29" s="209"/>
       <c r="H29" s="209"/>
-      <c r="I29" s="918" t="s">
+      <c r="I29" s="924" t="s">
         <v>217</v>
       </c>
-      <c r="J29" s="919"/>
-      <c r="K29" s="919"/>
-      <c r="L29" s="919"/>
-      <c r="M29" s="920"/>
+      <c r="J29" s="925"/>
+      <c r="K29" s="925"/>
+      <c r="L29" s="925"/>
+      <c r="M29" s="926"/>
       <c r="O29" s="209"/>
       <c r="P29" s="209"/>
       <c r="R29" s="209"/>
@@ -19901,15 +19901,15 @@
       </c>
       <c r="G30" s="209"/>
       <c r="H30" s="209"/>
-      <c r="I30" s="928" t="s">
+      <c r="I30" s="920" t="s">
         <v>212</v>
       </c>
-      <c r="J30" s="929"/>
-      <c r="K30" s="928" t="s">
+      <c r="J30" s="921"/>
+      <c r="K30" s="920" t="s">
         <v>213</v>
       </c>
-      <c r="L30" s="929"/>
-      <c r="M30" s="916" t="s">
+      <c r="L30" s="921"/>
+      <c r="M30" s="922" t="s">
         <v>214</v>
       </c>
       <c r="O30" s="209"/>
@@ -19945,7 +19945,7 @@
       <c r="L31" s="275" t="s">
         <v>216</v>
       </c>
-      <c r="M31" s="917"/>
+      <c r="M31" s="923"/>
       <c r="O31" s="209"/>
       <c r="P31" s="209"/>
       <c r="R31" s="209"/>
@@ -20112,12 +20112,12 @@
         <f>RSQ(D30:D32,B30:B32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D40" s="924" t="e">
+      <c r="D40" s="916" t="e">
         <f>IF(C40&lt;=0.95,"NO CONFORME","CONFORME")</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E40" s="925"/>
-      <c r="F40" s="926"/>
+      <c r="E40" s="917"/>
+      <c r="F40" s="918"/>
       <c r="G40" s="209"/>
       <c r="H40" s="257"/>
       <c r="I40" s="257"/>
@@ -20189,6 +20189,12 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="QbK/P4ukgbZU85pj93hV0ftn6ZZr2hJ3Xae2c00zbnGLirnsM7iT5h3St32dri55u5WTm1SV+UiG1Ty1N6MUfA==" saltValue="z/psz9/vsbYUqIhFhYyGLg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="M30:M31"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="I24:L24"/>
     <mergeCell ref="D40:F40"/>
     <mergeCell ref="I11:L11"/>
     <mergeCell ref="C11:H11"/>
@@ -20196,12 +20202,6 @@
     <mergeCell ref="I12:L12"/>
     <mergeCell ref="I30:J30"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="M30:M31"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:L3"/>
-    <mergeCell ref="I24:L24"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C12 I12" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -23277,18 +23277,18 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="953" t="s">
+      <c r="B19" s="959" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="953"/>
-      <c r="D19" s="953"/>
-      <c r="E19" s="953"/>
+      <c r="C19" s="959"/>
+      <c r="D19" s="959"/>
+      <c r="E19" s="959"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="328"/>
-      <c r="B20" s="958"/>
-      <c r="C20" s="958"/>
-      <c r="D20" s="958"/>
+      <c r="B20" s="953"/>
+      <c r="C20" s="953"/>
+      <c r="D20" s="953"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="236"/>
@@ -23339,20 +23339,20 @@
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="340"/>
-      <c r="B24" s="963" t="s">
+      <c r="B24" s="956" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="964"/>
-      <c r="D24" s="964"/>
-      <c r="E24" s="964"/>
-      <c r="F24" s="964"/>
-      <c r="G24" s="965"/>
-      <c r="H24" s="963" t="s">
+      <c r="C24" s="957"/>
+      <c r="D24" s="957"/>
+      <c r="E24" s="957"/>
+      <c r="F24" s="957"/>
+      <c r="G24" s="958"/>
+      <c r="H24" s="956" t="s">
         <v>144</v>
       </c>
-      <c r="I24" s="964"/>
-      <c r="J24" s="964"/>
-      <c r="K24" s="965"/>
+      <c r="I24" s="957"/>
+      <c r="J24" s="957"/>
+      <c r="K24" s="958"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="353" t="s">
@@ -23515,10 +23515,10 @@
       <c r="B29" s="330"/>
       <c r="C29" s="332"/>
       <c r="D29" s="330"/>
-      <c r="F29" s="958"/>
-      <c r="G29" s="958"/>
-      <c r="H29" s="958"/>
-      <c r="I29" s="958"/>
+      <c r="F29" s="953"/>
+      <c r="G29" s="953"/>
+      <c r="H29" s="953"/>
+      <c r="I29" s="953"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H30" s="350"/>
@@ -23526,17 +23526,17 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="328"/>
-      <c r="C31" s="959" t="s">
+      <c r="C31" s="963" t="s">
         <v>182</v>
       </c>
-      <c r="D31" s="960"/>
-      <c r="E31" s="961"/>
-      <c r="G31" s="957" t="s">
+      <c r="D31" s="964"/>
+      <c r="E31" s="965"/>
+      <c r="G31" s="955" t="s">
         <v>189</v>
       </c>
-      <c r="H31" s="957"/>
-      <c r="I31" s="957"/>
-      <c r="J31" s="957"/>
+      <c r="H31" s="955"/>
+      <c r="I31" s="955"/>
+      <c r="J31" s="955"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C32" s="335" t="s">
@@ -23552,7 +23552,7 @@
         <v>190</v>
       </c>
       <c r="H32" s="472">
-        <v>45485</v>
+        <v>45847</v>
       </c>
       <c r="I32" s="342">
         <v>7.3000000000000001E-3</v>
@@ -23562,7 +23562,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="962"/>
+      <c r="A33" s="954"/>
       <c r="C33" s="469">
         <v>1</v>
       </c>
@@ -23574,7 +23574,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="962"/>
+      <c r="A34" s="954"/>
       <c r="C34" s="469">
         <v>2</v>
       </c>
@@ -23586,7 +23586,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="962"/>
+      <c r="A35" s="954"/>
       <c r="C35" s="469">
         <v>3</v>
       </c>
@@ -23598,7 +23598,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="962"/>
+      <c r="A36" s="954"/>
       <c r="C36" s="469">
         <v>4</v>
       </c>
@@ -23610,7 +23610,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="954"/>
+      <c r="A37" s="960"/>
       <c r="C37" s="469">
         <v>5</v>
       </c>
@@ -23622,7 +23622,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="954"/>
+      <c r="A38" s="960"/>
       <c r="C38" s="469">
         <v>6</v>
       </c>
@@ -23634,7 +23634,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="954"/>
+      <c r="A39" s="960"/>
       <c r="C39" s="469">
         <v>7</v>
       </c>
@@ -23646,7 +23646,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="954"/>
+      <c r="A40" s="960"/>
       <c r="C40" s="469">
         <v>8</v>
       </c>
@@ -23801,21 +23801,21 @@
         <f>COUNT(C33:C52)</f>
         <v>20</v>
       </c>
-      <c r="C54" s="955" t="s">
+      <c r="C54" s="961" t="s">
         <v>186</v>
       </c>
-      <c r="D54" s="956"/>
+      <c r="D54" s="962"/>
       <c r="E54" s="582">
         <f>+STDEV(E33:E53)</f>
         <v>0.67082039324993703</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B55" s="957" t="s">
+      <c r="B55" s="955" t="s">
         <v>246</v>
       </c>
-      <c r="C55" s="957"/>
-      <c r="D55" s="957"/>
+      <c r="C55" s="955"/>
+      <c r="D55" s="955"/>
       <c r="E55" s="582">
         <f>E54/SQRT(B54)</f>
         <v>0.15000000000000002</v>
@@ -23824,17 +23824,17 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="H24:K24"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="A37:A40"/>
     <mergeCell ref="C54:D54"/>
     <mergeCell ref="B55:D55"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="C31:E31"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="H24:K24"/>
   </mergeCells>
   <conditionalFormatting sqref="E53">
     <cfRule type="cellIs" priority="1" stopIfTrue="1" operator="between">
@@ -25318,9 +25318,9 @@
       <c r="A2" s="329"/>
       <c r="G2" s="329"/>
       <c r="M2" s="328"/>
-      <c r="N2" s="958"/>
-      <c r="O2" s="958"/>
-      <c r="P2" s="958"/>
+      <c r="N2" s="953"/>
+      <c r="O2" s="953"/>
+      <c r="P2" s="953"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="329" t="s">
@@ -25329,7 +25329,7 @@
       <c r="G3" s="329" t="s">
         <v>327</v>
       </c>
-      <c r="M3" s="962"/>
+      <c r="M3" s="954"/>
       <c r="N3" s="656"/>
       <c r="O3" s="656"/>
       <c r="P3" s="656"/>
@@ -25347,7 +25347,7 @@
       <c r="H4" s="334">
         <v>46070</v>
       </c>
-      <c r="M4" s="962"/>
+      <c r="M4" s="954"/>
       <c r="N4" s="656"/>
       <c r="O4" s="657"/>
       <c r="P4" s="657"/>
@@ -25357,7 +25357,7 @@
       <c r="B5" s="658"/>
       <c r="G5" s="329"/>
       <c r="H5" s="658"/>
-      <c r="M5" s="962"/>
+      <c r="M5" s="954"/>
       <c r="N5" s="330"/>
       <c r="O5" s="330"/>
       <c r="P5" s="330"/>

</xml_diff>